<commit_message>
rerun model qwen3.5:9b RAG Base Model results generated
</commit_message>
<xml_diff>
--- a/results/qwen3_5_9b/comparison_SimpleRAG/SimpleRAG_consolidated.xlsx
+++ b/results/qwen3_5_9b/comparison_SimpleRAG/SimpleRAG_consolidated.xlsx
@@ -545,44 +545,46 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0.01010100960871342</v>
+        <v>0.179999995410889</v>
       </c>
       <c r="D2" t="n">
-        <v>7.188271943170174e-260</v>
+        <v>0.02185874490760725</v>
       </c>
       <c r="E2" t="n">
-        <v>0.3537169694900513</v>
+        <v>0.6043150424957275</v>
       </c>
       <c r="F2" t="n">
-        <v>-6.694999999999993</v>
+        <v>23.48171289241085</v>
       </c>
       <c r="G2" t="n">
-        <v>0.07379375591296121</v>
+        <v>0.651844843897824</v>
       </c>
       <c r="H2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J2" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J2" t="n">
+        <v>1</v>
+      </c>
       <c r="K2" t="n">
         <v>1</v>
       </c>
       <c r="L2" t="n">
-        <v>0.25</v>
+        <v>0.2857142857142857</v>
       </c>
       <c r="M2" t="n">
-        <v>0.1428571428571428</v>
+        <v>0.2622950819672131</v>
       </c>
       <c r="N2" t="n">
-        <v>76.47203207015991</v>
+        <v>160.1122732162476</v>
       </c>
       <c r="O2" t="n">
-        <v>1434.66015625</v>
+        <v>1439.83984375</v>
       </c>
       <c r="P2" t="n">
-        <v>10.4</v>
+        <v>11.1</v>
       </c>
       <c r="Q2" t="n">
         <v>0</v>
@@ -591,10 +593,10 @@
         <v>0</v>
       </c>
       <c r="S2" t="n">
-        <v>0.8389444351196289</v>
+        <v>1.101526260375977</v>
       </c>
       <c r="T2" t="n">
-        <v>75.63308262825012</v>
+        <v>159.0107429027557</v>
       </c>
       <c r="U2" t="n">
         <v>0</v>
@@ -610,19 +612,19 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0</v>
+        <v>0.1599999968000001</v>
       </c>
       <c r="D3" t="n">
-        <v>0</v>
+        <v>3.162429961676339e-155</v>
       </c>
       <c r="E3" t="n">
-        <v>0.4298741221427917</v>
+        <v>0.5548350214958191</v>
       </c>
       <c r="F3" t="n">
-        <v>-6.694999999999993</v>
+        <v>16.766847826087</v>
       </c>
       <c r="G3" t="n">
-        <v>0.7155963302752294</v>
+        <v>2.339449541284404</v>
       </c>
       <c r="H3" t="n">
         <v>0</v>
@@ -630,24 +632,26 @@
       <c r="I3" t="n">
         <v>0</v>
       </c>
-      <c r="J3" t="inlineStr"/>
+      <c r="J3" t="n">
+        <v>1</v>
+      </c>
       <c r="K3" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="L3" t="n">
-        <v>0.25</v>
+        <v>0.3225806451612903</v>
       </c>
       <c r="M3" t="n">
-        <v>0.1428571428571428</v>
+        <v>0.1208791208791209</v>
       </c>
       <c r="N3" t="n">
-        <v>1.984262704849243</v>
+        <v>365.7186002731323</v>
       </c>
       <c r="O3" t="n">
-        <v>1434.87109375</v>
+        <v>1440.5390625</v>
       </c>
       <c r="P3" t="n">
-        <v>17.1</v>
+        <v>15</v>
       </c>
       <c r="Q3" t="n">
         <v>0</v>
@@ -656,10 +660,10 @@
         <v>0</v>
       </c>
       <c r="S3" t="n">
-        <v>0.319493293762207</v>
+        <v>1.400856733322144</v>
       </c>
       <c r="T3" t="n">
-        <v>1.664765357971191</v>
+        <v>364.3177394866943</v>
       </c>
       <c r="U3" t="n">
         <v>0</v>
@@ -675,44 +679,46 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0</v>
+        <v>0.2396313323638217</v>
       </c>
       <c r="D4" t="n">
-        <v>0</v>
+        <v>0.003751756555926853</v>
       </c>
       <c r="E4" t="n">
-        <v>0.2991204261779785</v>
+        <v>0.6371692419052124</v>
       </c>
       <c r="F4" t="n">
-        <v>-6.694999999999993</v>
+        <v>31.87099483204136</v>
       </c>
       <c r="G4" t="n">
-        <v>0.08333333333333333</v>
+        <v>0.405982905982906</v>
       </c>
       <c r="H4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I4" t="n">
         <v>1</v>
       </c>
-      <c r="J4" t="inlineStr"/>
+      <c r="J4" t="n">
+        <v>1</v>
+      </c>
       <c r="K4" t="n">
         <v>0.5</v>
       </c>
       <c r="L4" t="n">
+        <v>0.4285714285714285</v>
+      </c>
+      <c r="M4" t="n">
         <v>0.25</v>
       </c>
-      <c r="M4" t="n">
-        <v>0.1428571428571428</v>
-      </c>
       <c r="N4" t="n">
-        <v>1.137856483459473</v>
+        <v>12.39716982841492</v>
       </c>
       <c r="O4" t="n">
-        <v>1435.0078125</v>
+        <v>1440.578125</v>
       </c>
       <c r="P4" t="n">
-        <v>14.1</v>
+        <v>12.2</v>
       </c>
       <c r="Q4" t="n">
         <v>0</v>
@@ -721,10 +727,10 @@
         <v>0</v>
       </c>
       <c r="S4" t="n">
-        <v>0.05013179779052734</v>
+        <v>1.236253499984741</v>
       </c>
       <c r="T4" t="n">
-        <v>1.087722063064575</v>
+        <v>11.16091394424438</v>
       </c>
       <c r="U4" t="n">
         <v>0</v>
@@ -740,44 +746,46 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0</v>
+        <v>0.2413793065776457</v>
       </c>
       <c r="D5" t="n">
-        <v>0</v>
+        <v>1.077201656108163e-79</v>
       </c>
       <c r="E5" t="n">
-        <v>0.2943938076496124</v>
+        <v>0.6558974385261536</v>
       </c>
       <c r="F5" t="n">
-        <v>-6.694999999999993</v>
+        <v>52.62126859504136</v>
       </c>
       <c r="G5" t="n">
-        <v>0.06382978723404255</v>
+        <v>0.3649754500818331</v>
       </c>
       <c r="H5" t="n">
-        <v>0</v>
+        <v>0.8</v>
       </c>
       <c r="I5" t="n">
         <v>1</v>
       </c>
-      <c r="J5" t="inlineStr"/>
+      <c r="J5" t="n">
+        <v>1</v>
+      </c>
       <c r="K5" t="n">
         <v>0</v>
       </c>
       <c r="L5" t="n">
-        <v>0.25</v>
+        <v>0.4406779661016949</v>
       </c>
       <c r="M5" t="n">
-        <v>0.1428571428571428</v>
+        <v>0.2682926829268293</v>
       </c>
       <c r="N5" t="n">
-        <v>1.754924535751343</v>
+        <v>10.72837734222412</v>
       </c>
       <c r="O5" t="n">
-        <v>1435.07421875</v>
+        <v>1441.78125</v>
       </c>
       <c r="P5" t="n">
-        <v>9.1</v>
+        <v>12.1</v>
       </c>
       <c r="Q5" t="n">
         <v>0</v>
@@ -786,10 +794,10 @@
         <v>0</v>
       </c>
       <c r="S5" t="n">
-        <v>0.05014634132385254</v>
+        <v>0.3296880722045898</v>
       </c>
       <c r="T5" t="n">
-        <v>1.704776048660278</v>
+        <v>10.398686170578</v>
       </c>
       <c r="U5" t="n">
         <v>0</v>
@@ -805,44 +813,46 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>0.01273885288652687</v>
+        <v>0.17592592175583</v>
       </c>
       <c r="D6" t="n">
-        <v>7.842246496009318e-255</v>
+        <v>5.513513681957571e-156</v>
       </c>
       <c r="E6" t="n">
-        <v>0.3298570215702057</v>
+        <v>0.6085430383682251</v>
       </c>
       <c r="F6" t="n">
-        <v>-6.694999999999993</v>
+        <v>45.97646464646465</v>
       </c>
       <c r="G6" t="n">
-        <v>0.0896551724137931</v>
+        <v>0.4367816091954023</v>
       </c>
       <c r="H6" t="n">
-        <v>0</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="I6" t="n">
         <v>1</v>
       </c>
-      <c r="J6" t="inlineStr"/>
+      <c r="J6" t="n">
+        <v>1</v>
+      </c>
       <c r="K6" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="L6" t="n">
-        <v>0.25</v>
+        <v>0.3541666666666667</v>
       </c>
       <c r="M6" t="n">
-        <v>0.1428571428571428</v>
+        <v>0.2134831460674157</v>
       </c>
       <c r="N6" t="n">
-        <v>1.332970142364502</v>
+        <v>13.05308818817139</v>
       </c>
       <c r="O6" t="n">
-        <v>1435.16015625</v>
+        <v>1441.79296875</v>
       </c>
       <c r="P6" t="n">
-        <v>8.9</v>
+        <v>14.2</v>
       </c>
       <c r="Q6" t="n">
         <v>0</v>
@@ -851,10 +861,10 @@
         <v>0</v>
       </c>
       <c r="S6" t="n">
-        <v>0.0514833927154541</v>
+        <v>0.2729661464691162</v>
       </c>
       <c r="T6" t="n">
-        <v>1.28148365020752</v>
+        <v>12.78011965751648</v>
       </c>
       <c r="U6" t="n">
         <v>0</v>
@@ -870,19 +880,19 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>0.004032257864935623</v>
+        <v>0.08598130690163334</v>
       </c>
       <c r="D7" t="n">
-        <v>0</v>
+        <v>3.813999754289355e-88</v>
       </c>
       <c r="E7" t="n">
-        <v>0.353213906288147</v>
+        <v>0.550951361656189</v>
       </c>
       <c r="F7" t="n">
-        <v>-6.694999999999993</v>
+        <v>15.92500000000004</v>
       </c>
       <c r="G7" t="n">
-        <v>0.02269421006691882</v>
+        <v>0.08961303462321792</v>
       </c>
       <c r="H7" t="n">
         <v>0</v>
@@ -890,24 +900,26 @@
       <c r="I7" t="n">
         <v>0</v>
       </c>
-      <c r="J7" t="inlineStr"/>
+      <c r="J7" t="n">
+        <v>0</v>
+      </c>
       <c r="K7" t="n">
         <v>0.5</v>
       </c>
       <c r="L7" t="n">
-        <v>0.25</v>
+        <v>0.2105263157894737</v>
       </c>
       <c r="M7" t="n">
-        <v>0.2</v>
+        <v>0.2063492063492064</v>
       </c>
       <c r="N7" t="n">
-        <v>1.759987354278564</v>
+        <v>13.98302745819092</v>
       </c>
       <c r="O7" t="n">
-        <v>1435.3125</v>
+        <v>1441.94140625</v>
       </c>
       <c r="P7" t="n">
-        <v>9.199999999999999</v>
+        <v>14.2</v>
       </c>
       <c r="Q7" t="n">
         <v>0</v>
@@ -916,10 +928,10 @@
         <v>0</v>
       </c>
       <c r="S7" t="n">
-        <v>0.08331394195556641</v>
+        <v>0.2783322334289551</v>
       </c>
       <c r="T7" t="n">
-        <v>1.676670551300049</v>
+        <v>13.70469331741333</v>
       </c>
       <c r="U7" t="n">
         <v>0</v>
@@ -935,44 +947,46 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>0</v>
+        <v>0.1880877702168808</v>
       </c>
       <c r="D8" t="n">
-        <v>0</v>
+        <v>3.782611663077085e-79</v>
       </c>
       <c r="E8" t="n">
-        <v>0.3415371477603912</v>
+        <v>0.5955166816711426</v>
       </c>
       <c r="F8" t="n">
-        <v>-6.694999999999993</v>
+        <v>33.44761904761904</v>
       </c>
       <c r="G8" t="n">
-        <v>0.05416666666666667</v>
+        <v>0.425</v>
       </c>
       <c r="H8" t="n">
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="I8" t="n">
-        <v>0</v>
-      </c>
-      <c r="J8" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J8" t="n">
+        <v>1</v>
+      </c>
       <c r="K8" t="n">
         <v>0.5</v>
       </c>
       <c r="L8" t="n">
-        <v>0.25</v>
+        <v>0.2682926829268293</v>
       </c>
       <c r="M8" t="n">
-        <v>0.06666666666666667</v>
+        <v>0.4214876033057851</v>
       </c>
       <c r="N8" t="n">
-        <v>1.224164962768555</v>
+        <v>28.58141660690308</v>
       </c>
       <c r="O8" t="n">
-        <v>1435.36328125</v>
+        <v>1442.04296875</v>
       </c>
       <c r="P8" t="n">
-        <v>9.1</v>
+        <v>14.3</v>
       </c>
       <c r="Q8" t="n">
         <v>0</v>
@@ -981,10 +995,10 @@
         <v>0</v>
       </c>
       <c r="S8" t="n">
-        <v>0.04852032661437988</v>
+        <v>0.237790584564209</v>
       </c>
       <c r="T8" t="n">
-        <v>1.175642251968384</v>
+        <v>28.34362387657166</v>
       </c>
       <c r="U8" t="n">
         <v>0</v>
@@ -1000,44 +1014,46 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>0.006993006649469429</v>
+        <v>0.1520467806947437</v>
       </c>
       <c r="D9" t="n">
-        <v>4.626996437597695e-283</v>
+        <v>4.184799915876941e-158</v>
       </c>
       <c r="E9" t="n">
-        <v>0.3237474858760834</v>
+        <v>0.6195626854896545</v>
       </c>
       <c r="F9" t="n">
-        <v>-6.694999999999993</v>
+        <v>33.65204113924054</v>
       </c>
       <c r="G9" t="n">
-        <v>0.04519119351100811</v>
+        <v>0.2195828505214369</v>
       </c>
       <c r="H9" t="n">
-        <v>0</v>
+        <v>0.375</v>
       </c>
       <c r="I9" t="n">
         <v>1</v>
       </c>
-      <c r="J9" t="inlineStr"/>
+      <c r="J9" t="n">
+        <v>1</v>
+      </c>
       <c r="K9" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="L9" t="n">
-        <v>0.25</v>
+        <v>0.4181818181818182</v>
       </c>
       <c r="M9" t="n">
-        <v>0.1428571428571428</v>
+        <v>0.1954022988505747</v>
       </c>
       <c r="N9" t="n">
-        <v>0.4575881958007812</v>
+        <v>12.63077235221863</v>
       </c>
       <c r="O9" t="n">
-        <v>1435.36328125</v>
+        <v>1442.16015625</v>
       </c>
       <c r="P9" t="n">
-        <v>8</v>
+        <v>14.3</v>
       </c>
       <c r="Q9" t="n">
         <v>0</v>
@@ -1046,10 +1062,10 @@
         <v>0</v>
       </c>
       <c r="S9" t="n">
-        <v>0.08756685256958008</v>
+        <v>0.2958860397338867</v>
       </c>
       <c r="T9" t="n">
-        <v>0.3700182437896729</v>
+        <v>12.33488368988037</v>
       </c>
       <c r="U9" t="n">
         <v>0</v>
@@ -1065,44 +1081,46 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>0</v>
+        <v>0.1733333300935556</v>
       </c>
       <c r="D10" t="n">
-        <v>0</v>
+        <v>1.587341920964993e-79</v>
       </c>
       <c r="E10" t="n">
-        <v>0.3335631489753723</v>
+        <v>0.5963821411132812</v>
       </c>
       <c r="F10" t="n">
-        <v>-6.694999999999993</v>
+        <v>43.19006787330318</v>
       </c>
       <c r="G10" t="n">
-        <v>0.05158730158730158</v>
+        <v>0.3108465608465609</v>
       </c>
       <c r="H10" t="n">
-        <v>0</v>
+        <v>0.3125</v>
       </c>
       <c r="I10" t="n">
-        <v>0</v>
-      </c>
-      <c r="J10" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J10" t="n">
+        <v>1</v>
+      </c>
       <c r="K10" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="L10" t="n">
-        <v>0.25</v>
+        <v>0.22</v>
       </c>
       <c r="M10" t="n">
-        <v>0.06666666666666667</v>
+        <v>0.24</v>
       </c>
       <c r="N10" t="n">
-        <v>0.4116129875183105</v>
+        <v>26.68319201469421</v>
       </c>
       <c r="O10" t="n">
-        <v>1435.44140625</v>
+        <v>1442.22265625</v>
       </c>
       <c r="P10" t="n">
-        <v>8.9</v>
+        <v>14.5</v>
       </c>
       <c r="Q10" t="n">
         <v>0</v>
@@ -1111,10 +1129,10 @@
         <v>0</v>
       </c>
       <c r="S10" t="n">
-        <v>0.04895162582397461</v>
+        <v>0.247819185256958</v>
       </c>
       <c r="T10" t="n">
-        <v>0.3626582622528076</v>
+        <v>26.43537044525146</v>
       </c>
       <c r="U10" t="n">
         <v>0</v>
@@ -1130,19 +1148,19 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>0.006756756424625656</v>
+        <v>0.124629077761361</v>
       </c>
       <c r="D11" t="n">
-        <v>3.199290466293744e-295</v>
+        <v>2.727136953450956e-157</v>
       </c>
       <c r="E11" t="n">
-        <v>0.312595933675766</v>
+        <v>0.5827984213829041</v>
       </c>
       <c r="F11" t="n">
-        <v>-6.694999999999993</v>
+        <v>64.90326271186441</v>
       </c>
       <c r="G11" t="n">
-        <v>0.04264625478403499</v>
+        <v>0.1864406779661017</v>
       </c>
       <c r="H11" t="n">
         <v>0</v>
@@ -1150,24 +1168,26 @@
       <c r="I11" t="n">
         <v>1</v>
       </c>
-      <c r="J11" t="inlineStr"/>
+      <c r="J11" t="n">
+        <v>1</v>
+      </c>
       <c r="K11" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="L11" t="n">
-        <v>0.25</v>
+        <v>0.4102564102564102</v>
       </c>
       <c r="M11" t="n">
-        <v>0.1428571428571428</v>
+        <v>0.3150684931506849</v>
       </c>
       <c r="N11" t="n">
-        <v>0.5006237030029297</v>
+        <v>19.38218235969543</v>
       </c>
       <c r="O11" t="n">
-        <v>1435.4453125</v>
+        <v>1442.26953125</v>
       </c>
       <c r="P11" t="n">
-        <v>10.4</v>
+        <v>13</v>
       </c>
       <c r="Q11" t="n">
         <v>0</v>
@@ -1176,10 +1196,10 @@
         <v>0</v>
       </c>
       <c r="S11" t="n">
-        <v>0.04920029640197754</v>
+        <v>0.2743501663208008</v>
       </c>
       <c r="T11" t="n">
-        <v>0.4514205455780029</v>
+        <v>19.10783004760742</v>
       </c>
       <c r="U11" t="n">
         <v>0</v>
@@ -1195,19 +1215,19 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>0</v>
+        <v>0.1049382693028883</v>
       </c>
       <c r="D12" t="n">
-        <v>0</v>
+        <v>1.048187222786645e-159</v>
       </c>
       <c r="E12" t="n">
-        <v>0.3295387625694275</v>
+        <v>0.5294414758682251</v>
       </c>
       <c r="F12" t="n">
-        <v>-6.694999999999993</v>
+        <v>28.63250000000002</v>
       </c>
       <c r="G12" t="n">
-        <v>0.04441913439635535</v>
+        <v>0.1588838268792711</v>
       </c>
       <c r="H12" t="n">
         <v>0</v>
@@ -1215,24 +1235,26 @@
       <c r="I12" t="n">
         <v>0</v>
       </c>
-      <c r="J12" t="inlineStr"/>
+      <c r="J12" t="n">
+        <v>1</v>
+      </c>
       <c r="K12" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="L12" t="n">
-        <v>0.25</v>
+        <v>0.3428571428571429</v>
       </c>
       <c r="M12" t="n">
-        <v>0.06666666666666667</v>
+        <v>0.1071428571428571</v>
       </c>
       <c r="N12" t="n">
-        <v>2.275068283081055</v>
+        <v>11.34494733810425</v>
       </c>
       <c r="O12" t="n">
-        <v>1435.484375</v>
+        <v>1442.31640625</v>
       </c>
       <c r="P12" t="n">
-        <v>10.5</v>
+        <v>13.6</v>
       </c>
       <c r="Q12" t="n">
         <v>0</v>
@@ -1241,10 +1263,10 @@
         <v>0</v>
       </c>
       <c r="S12" t="n">
-        <v>0.08544230461120605</v>
+        <v>0.2448604106903076</v>
       </c>
       <c r="T12" t="n">
-        <v>2.189622640609741</v>
+        <v>11.10008430480957</v>
       </c>
       <c r="U12" t="n">
         <v>0</v>
@@ -1260,44 +1282,46 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>0.006644517945718055</v>
+        <v>0.2347188224068484</v>
       </c>
       <c r="D13" t="n">
-        <v>1.737745674680046e-291</v>
+        <v>2.975131617077811e-156</v>
       </c>
       <c r="E13" t="n">
-        <v>0.3309608399868011</v>
+        <v>0.6754701137542725</v>
       </c>
       <c r="F13" t="n">
-        <v>-6.694999999999993</v>
+        <v>66.7609429280397</v>
       </c>
       <c r="G13" t="n">
-        <v>0.04323725055432372</v>
+        <v>0.3519955654101996</v>
       </c>
       <c r="H13" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="I13" t="n">
         <v>1</v>
       </c>
-      <c r="J13" t="inlineStr"/>
+      <c r="J13" t="n">
+        <v>1</v>
+      </c>
       <c r="K13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L13" t="n">
-        <v>0.25</v>
+        <v>0.303370786516854</v>
       </c>
       <c r="M13" t="n">
-        <v>0.1428571428571428</v>
+        <v>0.3137254901960784</v>
       </c>
       <c r="N13" t="n">
-        <v>0.4389102458953857</v>
+        <v>16.30511331558228</v>
       </c>
       <c r="O13" t="n">
-        <v>1435.59765625</v>
+        <v>1442.33984375</v>
       </c>
       <c r="P13" t="n">
-        <v>17.1</v>
+        <v>15.5</v>
       </c>
       <c r="Q13" t="n">
         <v>0</v>
@@ -1306,10 +1330,10 @@
         <v>0</v>
       </c>
       <c r="S13" t="n">
-        <v>0.04858088493347168</v>
+        <v>0.245225191116333</v>
       </c>
       <c r="T13" t="n">
-        <v>0.3903264999389648</v>
+        <v>16.05988502502441</v>
       </c>
       <c r="U13" t="n">
         <v>0</v>
@@ -1325,44 +1349,46 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>0</v>
+        <v>0.2222222190895062</v>
       </c>
       <c r="D14" t="n">
-        <v>0</v>
+        <v>0.002357693107793789</v>
       </c>
       <c r="E14" t="n">
-        <v>0.327696293592453</v>
+        <v>0.6467728018760681</v>
       </c>
       <c r="F14" t="n">
-        <v>-6.694999999999993</v>
+        <v>60.64184210526318</v>
       </c>
       <c r="G14" t="n">
-        <v>0.04333333333333333</v>
+        <v>0.2838888888888889</v>
       </c>
       <c r="H14" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="I14" t="n">
-        <v>0</v>
-      </c>
-      <c r="J14" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J14" t="n">
+        <v>1</v>
+      </c>
       <c r="K14" t="n">
-        <v>0.5</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="L14" t="n">
-        <v>0.25</v>
+        <v>0.2586206896551724</v>
       </c>
       <c r="M14" t="n">
-        <v>0.06666666666666667</v>
+        <v>0.3167701863354037</v>
       </c>
       <c r="N14" t="n">
-        <v>1.324690341949463</v>
+        <v>20.72277021408081</v>
       </c>
       <c r="O14" t="n">
-        <v>1435.640625</v>
+        <v>1442.33984375</v>
       </c>
       <c r="P14" t="n">
-        <v>18</v>
+        <v>12.7</v>
       </c>
       <c r="Q14" t="n">
         <v>0</v>
@@ -1371,10 +1397,10 @@
         <v>0</v>
       </c>
       <c r="S14" t="n">
-        <v>0.04912018775939941</v>
+        <v>0.2696521282196045</v>
       </c>
       <c r="T14" t="n">
-        <v>1.275567293167114</v>
+        <v>20.45311570167542</v>
       </c>
       <c r="U14" t="n">
         <v>0</v>
@@ -1390,44 +1416,46 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>0</v>
+        <v>0.2620689612366231</v>
       </c>
       <c r="D15" t="n">
-        <v>0</v>
+        <v>2.209311391872408e-155</v>
       </c>
       <c r="E15" t="n">
-        <v>0.3345783352851868</v>
+        <v>0.5793872475624084</v>
       </c>
       <c r="F15" t="n">
-        <v>-6.694999999999993</v>
+        <v>71.79366847826088</v>
       </c>
       <c r="G15" t="n">
-        <v>0.1569416498993964</v>
+        <v>0.6016096579476862</v>
       </c>
       <c r="H15" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="I15" t="n">
-        <v>0</v>
-      </c>
-      <c r="J15" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J15" t="n">
+        <v>1</v>
+      </c>
       <c r="K15" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="L15" t="n">
-        <v>0.25</v>
+        <v>0.3888888888888889</v>
       </c>
       <c r="M15" t="n">
-        <v>0.07692307692307693</v>
+        <v>0.2052980132450331</v>
       </c>
       <c r="N15" t="n">
-        <v>1.671306848526001</v>
+        <v>11.35493922233582</v>
       </c>
       <c r="O15" t="n">
-        <v>1435.6953125</v>
+        <v>1442.37109375</v>
       </c>
       <c r="P15" t="n">
-        <v>13.6</v>
+        <v>14.7</v>
       </c>
       <c r="Q15" t="n">
         <v>0</v>
@@ -1436,10 +1464,10 @@
         <v>0</v>
       </c>
       <c r="S15" t="n">
-        <v>0.04772257804870605</v>
+        <v>0.3284964561462402</v>
       </c>
       <c r="T15" t="n">
-        <v>1.623580455780029</v>
+        <v>11.02643966674805</v>
       </c>
       <c r="U15" t="n">
         <v>0</v>
@@ -1455,44 +1483,46 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>0</v>
+        <v>0.2090909042400828</v>
       </c>
       <c r="D16" t="n">
-        <v>0</v>
+        <v>7.595063987954255e-79</v>
       </c>
       <c r="E16" t="n">
-        <v>0.3279084861278534</v>
+        <v>0.6596572995185852</v>
       </c>
       <c r="F16" t="n">
-        <v>-6.694999999999993</v>
+        <v>43.52261871013468</v>
       </c>
       <c r="G16" t="n">
-        <v>0.1112696148359486</v>
+        <v>0.8316690442225392</v>
       </c>
       <c r="H16" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="I16" t="n">
-        <v>0</v>
-      </c>
-      <c r="J16" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J16" t="n">
+        <v>1</v>
+      </c>
       <c r="K16" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="L16" t="n">
-        <v>0.25</v>
+        <v>0.3181818181818182</v>
       </c>
       <c r="M16" t="n">
-        <v>0.07692307692307693</v>
+        <v>0.2405063291139241</v>
       </c>
       <c r="N16" t="n">
-        <v>0.5107827186584473</v>
+        <v>27.76741623878479</v>
       </c>
       <c r="O16" t="n">
-        <v>1435.7578125</v>
+        <v>1442.40234375</v>
       </c>
       <c r="P16" t="n">
-        <v>8.199999999999999</v>
+        <v>14.5</v>
       </c>
       <c r="Q16" t="n">
         <v>0</v>
@@ -1501,10 +1531,10 @@
         <v>0</v>
       </c>
       <c r="S16" t="n">
-        <v>0.05155420303344727</v>
+        <v>0.241471529006958</v>
       </c>
       <c r="T16" t="n">
-        <v>0.4592256546020508</v>
+        <v>27.52594113349915</v>
       </c>
       <c r="U16" t="n">
         <v>0</v>
@@ -1520,44 +1550,46 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>0</v>
+        <v>0.2629107934801296</v>
       </c>
       <c r="D17" t="n">
-        <v>0</v>
+        <v>1.169723085527137e-78</v>
       </c>
       <c r="E17" t="n">
-        <v>0.3277542293071747</v>
+        <v>0.6602102518081665</v>
       </c>
       <c r="F17" t="n">
-        <v>-6.694999999999993</v>
+        <v>52.49178571428573</v>
       </c>
       <c r="G17" t="n">
-        <v>0.1048387096774194</v>
+        <v>0.6559139784946236</v>
       </c>
       <c r="H17" t="n">
-        <v>0</v>
+        <v>0.1428571428571428</v>
       </c>
       <c r="I17" t="n">
-        <v>0</v>
-      </c>
-      <c r="J17" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J17" t="n">
+        <v>1</v>
+      </c>
       <c r="K17" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="L17" t="n">
+        <v>0.3859649122807017</v>
+      </c>
+      <c r="M17" t="n">
         <v>0.25</v>
       </c>
-      <c r="M17" t="n">
-        <v>0.07692307692307693</v>
-      </c>
       <c r="N17" t="n">
-        <v>1.133055925369263</v>
+        <v>16.28290700912476</v>
       </c>
       <c r="O17" t="n">
-        <v>1435.796875</v>
+        <v>1442.5703125</v>
       </c>
       <c r="P17" t="n">
-        <v>9.4</v>
+        <v>13.8</v>
       </c>
       <c r="Q17" t="n">
         <v>0</v>
@@ -1566,10 +1598,10 @@
         <v>0</v>
       </c>
       <c r="S17" t="n">
-        <v>0.05006504058837891</v>
+        <v>0.237107515335083</v>
       </c>
       <c r="T17" t="n">
-        <v>1.082988739013672</v>
+        <v>16.04579734802246</v>
       </c>
       <c r="U17" t="n">
         <v>0</v>
@@ -1585,44 +1617,46 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>0</v>
+        <v>0.2127659538821276</v>
       </c>
       <c r="D18" t="n">
-        <v>0</v>
+        <v>0.01009982552860134</v>
       </c>
       <c r="E18" t="n">
-        <v>0.3615763187408447</v>
+        <v>0.6351878046989441</v>
       </c>
       <c r="F18" t="n">
-        <v>-6.694999999999993</v>
+        <v>61.82779596376926</v>
       </c>
       <c r="G18" t="n">
-        <v>0.03037383177570093</v>
+        <v>0.2866043613707165</v>
       </c>
       <c r="H18" t="n">
-        <v>0</v>
+        <v>0.375</v>
       </c>
       <c r="I18" t="n">
-        <v>0</v>
-      </c>
-      <c r="J18" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J18" t="n">
+        <v>1</v>
+      </c>
       <c r="K18" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="L18" t="n">
-        <v>0.25</v>
+        <v>0.3061224489795918</v>
       </c>
       <c r="M18" t="n">
-        <v>0.1111111111111111</v>
+        <v>0.3181818181818182</v>
       </c>
       <c r="N18" t="n">
-        <v>0.8764533996582031</v>
+        <v>21.1650698184967</v>
       </c>
       <c r="O18" t="n">
-        <v>1435.796875</v>
+        <v>1442.6796875</v>
       </c>
       <c r="P18" t="n">
-        <v>8.800000000000001</v>
+        <v>14.1</v>
       </c>
       <c r="Q18" t="n">
         <v>0</v>
@@ -1631,10 +1665,10 @@
         <v>0</v>
       </c>
       <c r="S18" t="n">
-        <v>0.0492098331451416</v>
+        <v>0.2524657249450684</v>
       </c>
       <c r="T18" t="n">
-        <v>0.8272414207458496</v>
+        <v>20.91260123252869</v>
       </c>
       <c r="U18" t="n">
         <v>0</v>
@@ -1650,19 +1684,19 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>0</v>
+        <v>0.1774743999906813</v>
       </c>
       <c r="D19" t="n">
-        <v>0</v>
+        <v>1.023503195059246e-81</v>
       </c>
       <c r="E19" t="n">
-        <v>0.33333620429039</v>
+        <v>0.5886138081550598</v>
       </c>
       <c r="F19" t="n">
-        <v>-6.694999999999993</v>
+        <v>33.78275000000002</v>
       </c>
       <c r="G19" t="n">
-        <v>0.05141727092946605</v>
+        <v>0.2050098879367172</v>
       </c>
       <c r="H19" t="n">
         <v>0</v>
@@ -1670,24 +1704,26 @@
       <c r="I19" t="n">
         <v>0</v>
       </c>
-      <c r="J19" t="inlineStr"/>
+      <c r="J19" t="n">
+        <v>1</v>
+      </c>
       <c r="K19" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="L19" t="n">
-        <v>0.25</v>
+        <v>0.282051282051282</v>
       </c>
       <c r="M19" t="n">
-        <v>0.06666666666666667</v>
+        <v>0.140625</v>
       </c>
       <c r="N19" t="n">
-        <v>1.398208856582642</v>
+        <v>13.7309775352478</v>
       </c>
       <c r="O19" t="n">
-        <v>1435.796875</v>
+        <v>1442.765625</v>
       </c>
       <c r="P19" t="n">
-        <v>8.800000000000001</v>
+        <v>14.6</v>
       </c>
       <c r="Q19" t="n">
         <v>0</v>
@@ -1696,10 +1732,10 @@
         <v>0</v>
       </c>
       <c r="S19" t="n">
-        <v>0.09425926208496094</v>
+        <v>0.2454080581665039</v>
       </c>
       <c r="T19" t="n">
-        <v>1.303947448730469</v>
+        <v>13.48556685447693</v>
       </c>
       <c r="U19" t="n">
         <v>0</v>
@@ -1715,44 +1751,46 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>0.008032128120514206</v>
+        <v>0.1973333287873423</v>
       </c>
       <c r="D20" t="n">
-        <v>1.21304235279905e-268</v>
+        <v>6.643163136378773e-79</v>
       </c>
       <c r="E20" t="n">
-        <v>0.3513511121273041</v>
+        <v>0.6310942769050598</v>
       </c>
       <c r="F20" t="n">
-        <v>-6.694999999999993</v>
+        <v>50.72181343283583</v>
       </c>
       <c r="G20" t="n">
-        <v>0.05535841022001419</v>
+        <v>0.609652235628105</v>
       </c>
       <c r="H20" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="I20" t="n">
-        <v>0</v>
-      </c>
-      <c r="J20" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J20" t="n">
+        <v>1</v>
+      </c>
       <c r="K20" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="L20" t="n">
-        <v>0.25</v>
+        <v>0.2551020408163265</v>
       </c>
       <c r="M20" t="n">
-        <v>0.05882352941176471</v>
+        <v>0.3805309734513274</v>
       </c>
       <c r="N20" t="n">
-        <v>0.6292998790740967</v>
+        <v>27.69061994552612</v>
       </c>
       <c r="O20" t="n">
-        <v>1435.80078125</v>
+        <v>1442.86328125</v>
       </c>
       <c r="P20" t="n">
-        <v>8.4</v>
+        <v>14</v>
       </c>
       <c r="Q20" t="n">
         <v>0</v>
@@ -1761,10 +1799,10 @@
         <v>0</v>
       </c>
       <c r="S20" t="n">
-        <v>0.04818296432495117</v>
+        <v>0.2386364936828613</v>
       </c>
       <c r="T20" t="n">
-        <v>0.5811145305633545</v>
+        <v>27.45198035240173</v>
       </c>
       <c r="U20" t="n">
         <v>0</v>
@@ -1780,44 +1818,46 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>0</v>
+        <v>0.2379603360094376</v>
       </c>
       <c r="D21" t="n">
-        <v>0</v>
+        <v>0.005594593414339694</v>
       </c>
       <c r="E21" t="n">
-        <v>0.3501014113426208</v>
+        <v>0.573747992515564</v>
       </c>
       <c r="F21" t="n">
-        <v>-6.694999999999993</v>
+        <v>55.36715172413795</v>
       </c>
       <c r="G21" t="n">
-        <v>0.04419263456090652</v>
+        <v>0.3473087818696884</v>
       </c>
       <c r="H21" t="n">
-        <v>0</v>
+        <v>0.3</v>
       </c>
       <c r="I21" t="n">
-        <v>0</v>
-      </c>
-      <c r="J21" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J21" t="n">
+        <v>1</v>
+      </c>
       <c r="K21" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="L21" t="n">
-        <v>0.25</v>
+        <v>0.2716049382716049</v>
       </c>
       <c r="M21" t="n">
-        <v>0.01408450704225352</v>
+        <v>0.08653846153846154</v>
       </c>
       <c r="N21" t="n">
-        <v>1.240517139434814</v>
+        <v>14.50324845314026</v>
       </c>
       <c r="O21" t="n">
-        <v>1436.0703125</v>
+        <v>1442.87109375</v>
       </c>
       <c r="P21" t="n">
-        <v>8.699999999999999</v>
+        <v>13.9</v>
       </c>
       <c r="Q21" t="n">
         <v>0</v>
@@ -1826,10 +1866,10 @@
         <v>0</v>
       </c>
       <c r="S21" t="n">
-        <v>0.1213269233703613</v>
+        <v>0.2455160617828369</v>
       </c>
       <c r="T21" t="n">
-        <v>1.119187593460083</v>
+        <v>14.25773024559021</v>
       </c>
       <c r="U21" t="n">
         <v>0</v>
@@ -1845,19 +1885,19 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>0</v>
+        <v>0.1319444424153646</v>
       </c>
       <c r="D22" t="n">
-        <v>0</v>
+        <v>7.035603749466021e-84</v>
       </c>
       <c r="E22" t="n">
-        <v>0.3600354492664337</v>
+        <v>0.5146150588989258</v>
       </c>
       <c r="F22" t="n">
-        <v>-6.694999999999993</v>
+        <v>40.17500000000001</v>
       </c>
       <c r="G22" t="n">
-        <v>0.04727272727272727</v>
+        <v>0.1333333333333333</v>
       </c>
       <c r="H22" t="n">
         <v>0</v>
@@ -1865,24 +1905,26 @@
       <c r="I22" t="n">
         <v>0</v>
       </c>
-      <c r="J22" t="inlineStr"/>
+      <c r="J22" t="n">
+        <v>1</v>
+      </c>
       <c r="K22" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="L22" t="n">
-        <v>0.25</v>
+        <v>0.3461538461538461</v>
       </c>
       <c r="M22" t="n">
-        <v>0.05882352941176471</v>
+        <v>0.09090909090909091</v>
       </c>
       <c r="N22" t="n">
-        <v>1.365905046463013</v>
+        <v>15.0450713634491</v>
       </c>
       <c r="O22" t="n">
-        <v>1436.12109375</v>
+        <v>1442.87890625</v>
       </c>
       <c r="P22" t="n">
-        <v>8.9</v>
+        <v>13.9</v>
       </c>
       <c r="Q22" t="n">
         <v>0</v>
@@ -1891,10 +1933,10 @@
         <v>0</v>
       </c>
       <c r="S22" t="n">
-        <v>0.04926228523254395</v>
+        <v>0.2446608543395996</v>
       </c>
       <c r="T22" t="n">
-        <v>1.316640138626099</v>
+        <v>14.80040574073792</v>
       </c>
       <c r="U22" t="n">
         <v>0</v>
@@ -1910,44 +1952,46 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>0.005847952928251443</v>
+        <v>0.313167254985056</v>
       </c>
       <c r="D23" t="n">
-        <v>1.811128572821972e-307</v>
+        <v>1.159770719131815e-78</v>
       </c>
       <c r="E23" t="n">
-        <v>0.3535859286785126</v>
+        <v>0.6761953830718994</v>
       </c>
       <c r="F23" t="n">
-        <v>-6.694999999999993</v>
+        <v>29.33769841269844</v>
       </c>
       <c r="G23" t="n">
-        <v>0.0358291226458429</v>
+        <v>0.7005052824988516</v>
       </c>
       <c r="H23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I23" t="n">
-        <v>0</v>
-      </c>
-      <c r="J23" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J23" t="n">
+        <v>1</v>
+      </c>
       <c r="K23" t="n">
         <v>0.5</v>
       </c>
       <c r="L23" t="n">
-        <v>0.25</v>
+        <v>0.182741116751269</v>
       </c>
       <c r="M23" t="n">
-        <v>0.1111111111111111</v>
+        <v>0.7313432835820896</v>
       </c>
       <c r="N23" t="n">
-        <v>0.4961609840393066</v>
+        <v>36.80736088752747</v>
       </c>
       <c r="O23" t="n">
-        <v>1436.12890625</v>
+        <v>1442.890625</v>
       </c>
       <c r="P23" t="n">
-        <v>8.4</v>
+        <v>13.4</v>
       </c>
       <c r="Q23" t="n">
         <v>0</v>
@@ -1956,10 +2000,10 @@
         <v>0</v>
       </c>
       <c r="S23" t="n">
-        <v>0.04829525947570801</v>
+        <v>0.2396152019500732</v>
       </c>
       <c r="T23" t="n">
-        <v>0.4478635787963867</v>
+        <v>36.56774258613586</v>
       </c>
       <c r="U23" t="n">
         <v>0</v>
@@ -1975,44 +2019,46 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>0</v>
+        <v>0.2545454498850322</v>
       </c>
       <c r="D24" t="n">
-        <v>0</v>
+        <v>1.84425286803067e-155</v>
       </c>
       <c r="E24" t="n">
-        <v>0.3177126049995422</v>
+        <v>0.6434938311576843</v>
       </c>
       <c r="F24" t="n">
-        <v>-6.694999999999993</v>
+        <v>15.46001612903228</v>
       </c>
       <c r="G24" t="n">
-        <v>0.119815668202765</v>
+        <v>0.663594470046083</v>
       </c>
       <c r="H24" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I24" t="n">
-        <v>0</v>
-      </c>
-      <c r="J24" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J24" t="n">
+        <v>1</v>
+      </c>
       <c r="K24" t="n">
         <v>1</v>
       </c>
       <c r="L24" t="n">
-        <v>0.25</v>
+        <v>0.3061224489795918</v>
       </c>
       <c r="M24" t="n">
-        <v>0.09090909090909091</v>
+        <v>0.2024539877300613</v>
       </c>
       <c r="N24" t="n">
-        <v>1.187919616699219</v>
+        <v>14.4644033908844</v>
       </c>
       <c r="O24" t="n">
-        <v>1436.1328125</v>
+        <v>1442.90234375</v>
       </c>
       <c r="P24" t="n">
-        <v>9.1</v>
+        <v>13.9</v>
       </c>
       <c r="Q24" t="n">
         <v>0</v>
@@ -2021,10 +2067,10 @@
         <v>0</v>
       </c>
       <c r="S24" t="n">
-        <v>0.05022549629211426</v>
+        <v>0.2395079135894775</v>
       </c>
       <c r="T24" t="n">
-        <v>1.137691020965576</v>
+        <v>14.22489333152771</v>
       </c>
       <c r="U24" t="n">
         <v>0</v>
@@ -2040,44 +2086,46 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>0</v>
+        <v>0.2386363590399019</v>
       </c>
       <c r="D25" t="n">
-        <v>0</v>
+        <v>5.87773382411675e-79</v>
       </c>
       <c r="E25" t="n">
-        <v>0.3314136564731598</v>
+        <v>0.6541544795036316</v>
       </c>
       <c r="F25" t="n">
-        <v>-6.694999999999993</v>
+        <v>47.69637254901963</v>
       </c>
       <c r="G25" t="n">
-        <v>0.1176470588235294</v>
+        <v>0.5987933634992458</v>
       </c>
       <c r="H25" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I25" t="n">
-        <v>0</v>
-      </c>
-      <c r="J25" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J25" t="n">
+        <v>1</v>
+      </c>
       <c r="K25" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="L25" t="n">
+        <v>0.3846153846153846</v>
+      </c>
+      <c r="M25" t="n">
         <v>0.25</v>
       </c>
-      <c r="M25" t="n">
-        <v>0.1428571428571428</v>
-      </c>
       <c r="N25" t="n">
-        <v>0.4501781463623047</v>
+        <v>9.979879856109619</v>
       </c>
       <c r="O25" t="n">
-        <v>1436.1328125</v>
+        <v>1442.90625</v>
       </c>
       <c r="P25" t="n">
-        <v>12.2</v>
+        <v>14.9</v>
       </c>
       <c r="Q25" t="n">
         <v>0</v>
@@ -2086,10 +2134,10 @@
         <v>0</v>
       </c>
       <c r="S25" t="n">
-        <v>0.0893702507019043</v>
+        <v>0.2454454898834229</v>
       </c>
       <c r="T25" t="n">
-        <v>0.3608052730560303</v>
+        <v>9.734431982040405</v>
       </c>
       <c r="U25" t="n">
         <v>0</v>
@@ -2105,44 +2153,46 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>0</v>
+        <v>0.2624999951757813</v>
       </c>
       <c r="D26" t="n">
-        <v>0</v>
+        <v>9.346427289419537e-79</v>
       </c>
       <c r="E26" t="n">
-        <v>0.3261704742908478</v>
+        <v>0.6397182941436768</v>
       </c>
       <c r="F26" t="n">
-        <v>-6.694999999999993</v>
+        <v>22.86719230769236</v>
       </c>
       <c r="G26" t="n">
-        <v>0.1351819757365685</v>
+        <v>0.7435008665511266</v>
       </c>
       <c r="H26" t="n">
         <v>0</v>
       </c>
       <c r="I26" t="n">
-        <v>0</v>
-      </c>
-      <c r="J26" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J26" t="n">
+        <v>1</v>
+      </c>
       <c r="K26" t="n">
         <v>0.5</v>
       </c>
       <c r="L26" t="n">
-        <v>0.25</v>
+        <v>0.2307692307692308</v>
       </c>
       <c r="M26" t="n">
-        <v>0.1428571428571428</v>
+        <v>0.2771084337349398</v>
       </c>
       <c r="N26" t="n">
-        <v>1.510486841201782</v>
+        <v>8.834078311920166</v>
       </c>
       <c r="O26" t="n">
-        <v>1436.19921875</v>
+        <v>1442.9921875</v>
       </c>
       <c r="P26" t="n">
-        <v>18.2</v>
+        <v>12.4</v>
       </c>
       <c r="Q26" t="n">
         <v>0</v>
@@ -2151,10 +2201,10 @@
         <v>0</v>
       </c>
       <c r="S26" t="n">
-        <v>0.04884696006774902</v>
+        <v>0.2767970561981201</v>
       </c>
       <c r="T26" t="n">
-        <v>1.461637735366821</v>
+        <v>8.557279109954834</v>
       </c>
       <c r="U26" t="n">
         <v>0</v>
@@ -2170,44 +2220,46 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>0</v>
+        <v>0.2553191445523993</v>
       </c>
       <c r="D27" t="n">
-        <v>0</v>
+        <v>3.970998524709027e-79</v>
       </c>
       <c r="E27" t="n">
-        <v>0.3252985775470734</v>
+        <v>0.6008229851722717</v>
       </c>
       <c r="F27" t="n">
-        <v>-6.694999999999993</v>
+        <v>35.57723837209303</v>
       </c>
       <c r="G27" t="n">
-        <v>0.106703146374829</v>
+        <v>0.53077975376197</v>
       </c>
       <c r="H27" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I27" t="n">
-        <v>0</v>
-      </c>
-      <c r="J27" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J27" t="n">
+        <v>1</v>
+      </c>
       <c r="K27" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L27" t="n">
-        <v>0.25</v>
+        <v>0.26</v>
       </c>
       <c r="M27" t="n">
-        <v>0.1428571428571428</v>
+        <v>0.2405063291139241</v>
       </c>
       <c r="N27" t="n">
-        <v>1.326744079589844</v>
+        <v>10.23827743530273</v>
       </c>
       <c r="O27" t="n">
-        <v>1436.20703125</v>
+        <v>1443.12109375</v>
       </c>
       <c r="P27" t="n">
-        <v>18.4</v>
+        <v>15</v>
       </c>
       <c r="Q27" t="n">
         <v>0</v>
@@ -2216,10 +2268,10 @@
         <v>0</v>
       </c>
       <c r="S27" t="n">
-        <v>0.04909896850585938</v>
+        <v>0.2445876598358154</v>
       </c>
       <c r="T27" t="n">
-        <v>1.277642488479614</v>
+        <v>9.993687391281128</v>
       </c>
       <c r="U27" t="n">
         <v>0</v>
@@ -2235,44 +2287,46 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>0</v>
+        <v>0.2699386460536716</v>
       </c>
       <c r="D28" t="n">
-        <v>0</v>
+        <v>3.206501399135887e-79</v>
       </c>
       <c r="E28" t="n">
-        <v>0.3308320045471191</v>
+        <v>0.5576639771461487</v>
       </c>
       <c r="F28" t="n">
-        <v>-6.694999999999993</v>
+        <v>50.92565217391305</v>
       </c>
       <c r="G28" t="n">
-        <v>0.1181818181818182</v>
+        <v>0.4575757575757576</v>
       </c>
       <c r="H28" t="n">
         <v>0</v>
       </c>
       <c r="I28" t="n">
-        <v>0</v>
-      </c>
-      <c r="J28" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J28" t="n">
+        <v>1</v>
+      </c>
       <c r="K28" t="n">
         <v>1</v>
       </c>
       <c r="L28" t="n">
-        <v>0.25</v>
+        <v>0.3170731707317073</v>
       </c>
       <c r="M28" t="n">
-        <v>0.1428571428571428</v>
+        <v>0.1891891891891892</v>
       </c>
       <c r="N28" t="n">
-        <v>2.467652797698975</v>
+        <v>6.928074359893799</v>
       </c>
       <c r="O28" t="n">
-        <v>1436.2109375</v>
+        <v>1443.16015625</v>
       </c>
       <c r="P28" t="n">
-        <v>9</v>
+        <v>11.4</v>
       </c>
       <c r="Q28" t="n">
         <v>0</v>
@@ -2281,10 +2335,10 @@
         <v>0</v>
       </c>
       <c r="S28" t="n">
-        <v>0.05246353149414062</v>
+        <v>0.2437715530395508</v>
       </c>
       <c r="T28" t="n">
-        <v>2.415187120437622</v>
+        <v>6.684297561645508</v>
       </c>
       <c r="U28" t="n">
         <v>0</v>
@@ -2300,44 +2354,46 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>0</v>
+        <v>0.2598870006766894</v>
       </c>
       <c r="D29" t="n">
-        <v>0</v>
+        <v>1.171572819558805e-78</v>
       </c>
       <c r="E29" t="n">
-        <v>0.3268276154994965</v>
+        <v>0.6349772810935974</v>
       </c>
       <c r="F29" t="n">
-        <v>-6.694999999999993</v>
+        <v>14.28452702702705</v>
       </c>
       <c r="G29" t="n">
-        <v>0.1354166666666667</v>
+        <v>0.8888888888888888</v>
       </c>
       <c r="H29" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I29" t="n">
-        <v>0</v>
-      </c>
-      <c r="J29" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J29" t="n">
+        <v>1</v>
+      </c>
       <c r="K29" t="n">
         <v>0.5</v>
       </c>
       <c r="L29" t="n">
-        <v>0.25</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="M29" t="n">
-        <v>0.1428571428571428</v>
+        <v>0.358974358974359</v>
       </c>
       <c r="N29" t="n">
-        <v>0.5193507671356201</v>
+        <v>8.439210891723633</v>
       </c>
       <c r="O29" t="n">
-        <v>1436.2109375</v>
+        <v>1443.2265625</v>
       </c>
       <c r="P29" t="n">
-        <v>9.1</v>
+        <v>12.5</v>
       </c>
       <c r="Q29" t="n">
         <v>0</v>
@@ -2346,10 +2402,10 @@
         <v>0</v>
       </c>
       <c r="S29" t="n">
-        <v>0.04853558540344238</v>
+        <v>0.2376666069030762</v>
       </c>
       <c r="T29" t="n">
-        <v>0.4708130359649658</v>
+        <v>8.201541900634766</v>
       </c>
       <c r="U29" t="n">
         <v>0</v>
@@ -2365,44 +2421,46 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>0</v>
+        <v>0.1052631558067867</v>
       </c>
       <c r="D30" t="n">
-        <v>0</v>
+        <v>1.731819436118073e-155</v>
       </c>
       <c r="E30" t="n">
-        <v>0.4468841254711151</v>
+        <v>0.5131526589393616</v>
       </c>
       <c r="F30" t="n">
-        <v>-6.694999999999993</v>
+        <v>59.263688172043</v>
       </c>
       <c r="G30" t="n">
-        <v>0.78</v>
+        <v>4.76</v>
       </c>
       <c r="H30" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I30" t="n">
-        <v>0</v>
-      </c>
-      <c r="J30" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J30" t="n">
+        <v>1</v>
+      </c>
       <c r="K30" t="n">
         <v>1</v>
       </c>
       <c r="L30" t="n">
-        <v>0.25</v>
+        <v>0.3148148148148148</v>
       </c>
       <c r="M30" t="n">
-        <v>0.07692307692307693</v>
+        <v>0.2352941176470588</v>
       </c>
       <c r="N30" t="n">
-        <v>0.4102785587310791</v>
+        <v>13.08601450920105</v>
       </c>
       <c r="O30" t="n">
-        <v>1436.2109375</v>
+        <v>1443.3125</v>
       </c>
       <c r="P30" t="n">
-        <v>8.1</v>
+        <v>14.4</v>
       </c>
       <c r="Q30" t="n">
         <v>0</v>
@@ -2411,10 +2469,10 @@
         <v>0</v>
       </c>
       <c r="S30" t="n">
-        <v>0.04793906211853027</v>
+        <v>0.2410788536071777</v>
       </c>
       <c r="T30" t="n">
-        <v>0.3623368740081787</v>
+        <v>12.8449330329895</v>
       </c>
       <c r="U30" t="n">
         <v>0</v>
@@ -2430,44 +2488,46 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>0</v>
+        <v>0.1282051261637081</v>
       </c>
       <c r="D31" t="n">
-        <v>0</v>
+        <v>1.97145351198676e-155</v>
       </c>
       <c r="E31" t="n">
-        <v>0.4375941157341003</v>
+        <v>0.5361713171005249</v>
       </c>
       <c r="F31" t="n">
-        <v>-6.694999999999993</v>
+        <v>65.55811904761907</v>
       </c>
       <c r="G31" t="n">
-        <v>0.7572815533980582</v>
+        <v>4.456310679611651</v>
       </c>
       <c r="H31" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I31" t="n">
-        <v>0</v>
-      </c>
-      <c r="J31" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J31" t="n">
+        <v>1</v>
+      </c>
       <c r="K31" t="n">
         <v>1</v>
       </c>
       <c r="L31" t="n">
-        <v>0.25</v>
+        <v>0.375</v>
       </c>
       <c r="M31" t="n">
-        <v>0.07692307692307693</v>
+        <v>0.2307692307692308</v>
       </c>
       <c r="N31" t="n">
-        <v>0.4380490779876709</v>
+        <v>12.59663462638855</v>
       </c>
       <c r="O31" t="n">
-        <v>1436.2109375</v>
+        <v>1443.32421875</v>
       </c>
       <c r="P31" t="n">
-        <v>8.5</v>
+        <v>14.2</v>
       </c>
       <c r="Q31" t="n">
         <v>0</v>
@@ -2476,10 +2536,10 @@
         <v>0</v>
       </c>
       <c r="S31" t="n">
-        <v>0.04803729057312012</v>
+        <v>0.2400929927825928</v>
       </c>
       <c r="T31" t="n">
-        <v>0.3899977207183838</v>
+        <v>12.35653877258301</v>
       </c>
       <c r="U31" t="n">
         <v>0</v>
@@ -2495,44 +2555,46 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>0</v>
+        <v>0.1204819257773262</v>
       </c>
       <c r="D32" t="n">
-        <v>0</v>
+        <v>1.867555914367928e-155</v>
       </c>
       <c r="E32" t="n">
-        <v>0.4345121085643768</v>
+        <v>0.5348336100578308</v>
       </c>
       <c r="F32" t="n">
-        <v>-6.694999999999993</v>
+        <v>48.09089285714288</v>
       </c>
       <c r="G32" t="n">
-        <v>0.78</v>
+        <v>4.78</v>
       </c>
       <c r="H32" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I32" t="n">
-        <v>0</v>
-      </c>
-      <c r="J32" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J32" t="n">
+        <v>1</v>
+      </c>
       <c r="K32" t="n">
-        <v>1</v>
+        <v>0.75</v>
       </c>
       <c r="L32" t="n">
-        <v>0.25</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="M32" t="n">
-        <v>0.07692307692307693</v>
+        <v>0.2265193370165746</v>
       </c>
       <c r="N32" t="n">
-        <v>1.381005048751831</v>
+        <v>14.94927358627319</v>
       </c>
       <c r="O32" t="n">
-        <v>1436.2109375</v>
+        <v>1443.32421875</v>
       </c>
       <c r="P32" t="n">
-        <v>9.300000000000001</v>
+        <v>12.6</v>
       </c>
       <c r="Q32" t="n">
         <v>0</v>
@@ -2541,10 +2603,10 @@
         <v>0</v>
       </c>
       <c r="S32" t="n">
-        <v>0.04758119583129883</v>
+        <v>0.2361922264099121</v>
       </c>
       <c r="T32" t="n">
-        <v>1.333421230316162</v>
+        <v>14.71307873725891</v>
       </c>
       <c r="U32" t="n">
         <v>0</v>
@@ -2560,44 +2622,46 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>0</v>
+        <v>0.2205882305374136</v>
       </c>
       <c r="D33" t="n">
-        <v>0</v>
+        <v>0.02509047081322424</v>
       </c>
       <c r="E33" t="n">
-        <v>0.4005701541900635</v>
+        <v>0.6044853925704956</v>
       </c>
       <c r="F33" t="n">
-        <v>-6.694999999999993</v>
+        <v>61.90204678362574</v>
       </c>
       <c r="G33" t="n">
-        <v>0.2160664819944598</v>
+        <v>1.556786703601108</v>
       </c>
       <c r="H33" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I33" t="n">
-        <v>0</v>
-      </c>
-      <c r="J33" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J33" t="n">
+        <v>1</v>
+      </c>
       <c r="K33" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="L33" t="n">
-        <v>0.25</v>
+        <v>0.4347826086956522</v>
       </c>
       <c r="M33" t="n">
-        <v>0.09090909090909091</v>
+        <v>0.281437125748503</v>
       </c>
       <c r="N33" t="n">
-        <v>2.106777667999268</v>
+        <v>17.28743410110474</v>
       </c>
       <c r="O33" t="n">
-        <v>1436.296875</v>
+        <v>1443.33984375</v>
       </c>
       <c r="P33" t="n">
-        <v>9</v>
+        <v>15.3</v>
       </c>
       <c r="Q33" t="n">
         <v>0</v>
@@ -2606,10 +2670,10 @@
         <v>0</v>
       </c>
       <c r="S33" t="n">
-        <v>0.05308246612548828</v>
+        <v>0.2429637908935547</v>
       </c>
       <c r="T33" t="n">
-        <v>2.053693056106567</v>
+        <v>17.04446792602539</v>
       </c>
       <c r="U33" t="n">
         <v>0</v>
@@ -2625,44 +2689,46 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>0</v>
+        <v>0.1808510591557267</v>
       </c>
       <c r="D34" t="n">
-        <v>0</v>
+        <v>2.075505785857712e-155</v>
       </c>
       <c r="E34" t="n">
-        <v>0.3832495212554932</v>
+        <v>0.5973866581916809</v>
       </c>
       <c r="F34" t="n">
-        <v>-6.694999999999993</v>
+        <v>66.15478571428574</v>
       </c>
       <c r="G34" t="n">
-        <v>0.1133720930232558</v>
+        <v>0.6540697674418605</v>
       </c>
       <c r="H34" t="n">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="I34" t="n">
-        <v>0</v>
-      </c>
-      <c r="J34" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J34" t="n">
+        <v>1</v>
+      </c>
       <c r="K34" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="L34" t="n">
-        <v>0.25</v>
+        <v>0.3387096774193548</v>
       </c>
       <c r="M34" t="n">
-        <v>0.1428571428571428</v>
+        <v>0.2631578947368421</v>
       </c>
       <c r="N34" t="n">
-        <v>1.582678318023682</v>
+        <v>17.31186532974243</v>
       </c>
       <c r="O34" t="n">
-        <v>1436.31640625</v>
+        <v>1443.3515625</v>
       </c>
       <c r="P34" t="n">
-        <v>8.9</v>
+        <v>14.1</v>
       </c>
       <c r="Q34" t="n">
         <v>0</v>
@@ -2671,10 +2737,10 @@
         <v>0</v>
       </c>
       <c r="S34" t="n">
-        <v>0.04851651191711426</v>
+        <v>0.2443737983703613</v>
       </c>
       <c r="T34" t="n">
-        <v>1.534159183502197</v>
+        <v>17.06748843193054</v>
       </c>
       <c r="U34" t="n">
         <v>0</v>
@@ -2690,44 +2756,46 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>0</v>
+        <v>0.3696969649092746</v>
       </c>
       <c r="D35" t="n">
-        <v>0</v>
+        <v>0.06019347783543957</v>
       </c>
       <c r="E35" t="n">
-        <v>0.3523319959640503</v>
+        <v>0.6811069846153259</v>
       </c>
       <c r="F35" t="n">
-        <v>-6.694999999999993</v>
+        <v>45.93392717086837</v>
       </c>
       <c r="G35" t="n">
-        <v>0.06830122591943957</v>
+        <v>0.6611208406304728</v>
       </c>
       <c r="H35" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I35" t="n">
-        <v>0</v>
-      </c>
-      <c r="J35" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J35" t="n">
+        <v>1</v>
+      </c>
       <c r="K35" t="n">
         <v>1</v>
       </c>
       <c r="L35" t="n">
-        <v>0.25</v>
+        <v>0.3505154639175257</v>
       </c>
       <c r="M35" t="n">
-        <v>0.07692307692307693</v>
+        <v>0.4262295081967214</v>
       </c>
       <c r="N35" t="n">
-        <v>2.130998134613037</v>
+        <v>18.00968790054321</v>
       </c>
       <c r="O35" t="n">
-        <v>1436.421875</v>
+        <v>1443.3515625</v>
       </c>
       <c r="P35" t="n">
-        <v>13.7</v>
+        <v>13.1</v>
       </c>
       <c r="Q35" t="n">
         <v>0</v>
@@ -2736,10 +2804,10 @@
         <v>0</v>
       </c>
       <c r="S35" t="n">
-        <v>0.04872703552246094</v>
+        <v>0.2391109466552734</v>
       </c>
       <c r="T35" t="n">
-        <v>2.082268238067627</v>
+        <v>17.77057456970215</v>
       </c>
       <c r="U35" t="n">
         <v>0</v>
@@ -2755,44 +2823,46 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>0</v>
+        <v>0.2424242376283033</v>
       </c>
       <c r="D36" t="n">
-        <v>0</v>
+        <v>1.190965541157402e-78</v>
       </c>
       <c r="E36" t="n">
-        <v>0.3204767107963562</v>
+        <v>0.6990688443183899</v>
       </c>
       <c r="F36" t="n">
-        <v>-6.694999999999993</v>
+        <v>50.22437500000001</v>
       </c>
       <c r="G36" t="n">
-        <v>0.1236133122028526</v>
+        <v>0.8145800316957211</v>
       </c>
       <c r="H36" t="n">
         <v>0</v>
       </c>
       <c r="I36" t="n">
-        <v>0</v>
-      </c>
-      <c r="J36" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J36" t="n">
+        <v>1</v>
+      </c>
       <c r="K36" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="L36" t="n">
-        <v>0.25</v>
+        <v>0.3220338983050847</v>
       </c>
       <c r="M36" t="n">
-        <v>0.07692307692307693</v>
+        <v>0.3061224489795918</v>
       </c>
       <c r="N36" t="n">
-        <v>2.697059631347656</v>
+        <v>14.74432563781738</v>
       </c>
       <c r="O36" t="n">
-        <v>1436.53515625</v>
+        <v>1443.4453125</v>
       </c>
       <c r="P36" t="n">
-        <v>15.8</v>
+        <v>15.1</v>
       </c>
       <c r="Q36" t="n">
         <v>0</v>
@@ -2801,10 +2871,10 @@
         <v>0</v>
       </c>
       <c r="S36" t="n">
-        <v>0.05309915542602539</v>
+        <v>0.2454111576080322</v>
       </c>
       <c r="T36" t="n">
-        <v>2.643957614898682</v>
+        <v>14.49891138076782</v>
       </c>
       <c r="U36" t="n">
         <v>0</v>
@@ -2820,44 +2890,46 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>0</v>
+        <v>0.1089108875718068</v>
       </c>
       <c r="D37" t="n">
-        <v>0</v>
+        <v>3.996388526558475e-156</v>
       </c>
       <c r="E37" t="n">
-        <v>0.3582548201084137</v>
+        <v>0.5503356456756592</v>
       </c>
       <c r="F37" t="n">
-        <v>-6.694999999999993</v>
+        <v>28.04540140845072</v>
       </c>
       <c r="G37" t="n">
-        <v>0.08271474019088017</v>
+        <v>0.3435843054082715</v>
       </c>
       <c r="H37" t="n">
-        <v>0</v>
+        <v>0.1666666666666667</v>
       </c>
       <c r="I37" t="n">
-        <v>0</v>
-      </c>
-      <c r="J37" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J37" t="n">
+        <v>1</v>
+      </c>
       <c r="K37" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="L37" t="n">
-        <v>0.25</v>
+        <v>0.3846153846153846</v>
       </c>
       <c r="M37" t="n">
-        <v>0.1428571428571428</v>
+        <v>0.2553191489361702</v>
       </c>
       <c r="N37" t="n">
-        <v>0.525054931640625</v>
+        <v>18.94883227348328</v>
       </c>
       <c r="O37" t="n">
-        <v>1436.5546875</v>
+        <v>1443.4453125</v>
       </c>
       <c r="P37" t="n">
-        <v>9.800000000000001</v>
+        <v>13.8</v>
       </c>
       <c r="Q37" t="n">
         <v>0</v>
@@ -2866,10 +2938,10 @@
         <v>0</v>
       </c>
       <c r="S37" t="n">
-        <v>0.05364584922790527</v>
+        <v>0.281712532043457</v>
       </c>
       <c r="T37" t="n">
-        <v>0.4714062213897705</v>
+        <v>18.66711640357971</v>
       </c>
       <c r="U37" t="n">
         <v>0</v>
@@ -2885,44 +2957,46 @@
         </is>
       </c>
       <c r="C38" t="n">
-        <v>0</v>
+        <v>0.2068965470649617</v>
       </c>
       <c r="D38" t="n">
-        <v>0</v>
+        <v>2.179480756627313e-155</v>
       </c>
       <c r="E38" t="n">
-        <v>0.3565259277820587</v>
+        <v>0.5841172337532043</v>
       </c>
       <c r="F38" t="n">
-        <v>-6.694999999999993</v>
+        <v>36.20016806722691</v>
       </c>
       <c r="G38" t="n">
-        <v>0.1009055627425614</v>
+        <v>0.6015523932729625</v>
       </c>
       <c r="H38" t="n">
         <v>0</v>
       </c>
       <c r="I38" t="n">
-        <v>0</v>
-      </c>
-      <c r="J38" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J38" t="n">
+        <v>1</v>
+      </c>
       <c r="K38" t="n">
-        <v>0.5</v>
+        <v>0.925</v>
       </c>
       <c r="L38" t="n">
-        <v>0.25</v>
+        <v>0.2580645161290323</v>
       </c>
       <c r="M38" t="n">
-        <v>0.1111111111111111</v>
+        <v>0.3658536585365854</v>
       </c>
       <c r="N38" t="n">
-        <v>0.2687962055206299</v>
+        <v>17.63683772087097</v>
       </c>
       <c r="O38" t="n">
-        <v>1436.5546875</v>
+        <v>1443.56640625</v>
       </c>
       <c r="P38" t="n">
-        <v>8</v>
+        <v>14.1</v>
       </c>
       <c r="Q38" t="n">
         <v>0</v>
@@ -2931,10 +3005,10 @@
         <v>0</v>
       </c>
       <c r="S38" t="n">
-        <v>0.06898164749145508</v>
+        <v>0.2465879917144775</v>
       </c>
       <c r="T38" t="n">
-        <v>0.199812650680542</v>
+        <v>17.3902473449707</v>
       </c>
       <c r="U38" t="n">
         <v>0</v>
@@ -2950,44 +3024,46 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>0</v>
+        <v>0.2587064627063687</v>
       </c>
       <c r="D39" t="n">
-        <v>0</v>
+        <v>0.02459307181097702</v>
       </c>
       <c r="E39" t="n">
-        <v>0.3533079922199249</v>
+        <v>0.6409978270530701</v>
       </c>
       <c r="F39" t="n">
-        <v>-6.694999999999993</v>
+        <v>41.64287439613528</v>
       </c>
       <c r="G39" t="n">
-        <v>0.1150442477876106</v>
+        <v>0.855457227138643</v>
       </c>
       <c r="H39" t="n">
-        <v>0</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="I39" t="n">
-        <v>0</v>
-      </c>
-      <c r="J39" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J39" t="n">
+        <v>0</v>
+      </c>
       <c r="K39" t="n">
         <v>1</v>
       </c>
       <c r="L39" t="n">
-        <v>0.25</v>
+        <v>0.3461538461538461</v>
       </c>
       <c r="M39" t="n">
-        <v>0.05882352941176471</v>
+        <v>0.2424242424242424</v>
       </c>
       <c r="N39" t="n">
-        <v>0.4204061031341553</v>
+        <v>14.06314754486084</v>
       </c>
       <c r="O39" t="n">
-        <v>1436.5625</v>
+        <v>1443.6015625</v>
       </c>
       <c r="P39" t="n">
-        <v>8.5</v>
+        <v>14.3</v>
       </c>
       <c r="Q39" t="n">
         <v>0</v>
@@ -2996,10 +3072,10 @@
         <v>0</v>
       </c>
       <c r="S39" t="n">
-        <v>0.05163478851318359</v>
+        <v>0.2527048587799072</v>
       </c>
       <c r="T39" t="n">
-        <v>0.3687689304351807</v>
+        <v>13.81043791770935</v>
       </c>
       <c r="U39" t="n">
         <v>0</v>
@@ -3015,44 +3091,46 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>0</v>
+        <v>0.3399209438528957</v>
       </c>
       <c r="D40" t="n">
-        <v>0</v>
+        <v>0.0315443883087062</v>
       </c>
       <c r="E40" t="n">
-        <v>0.2973054349422455</v>
+        <v>0.6457474827766418</v>
       </c>
       <c r="F40" t="n">
-        <v>-6.694999999999993</v>
+        <v>49.31608241758244</v>
       </c>
       <c r="G40" t="n">
-        <v>0.08590308370044053</v>
+        <v>0.6806167400881057</v>
       </c>
       <c r="H40" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I40" t="n">
         <v>1</v>
       </c>
-      <c r="J40" t="inlineStr"/>
+      <c r="J40" t="n">
+        <v>1</v>
+      </c>
       <c r="K40" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="L40" t="n">
-        <v>0.25</v>
+        <v>0.325</v>
       </c>
       <c r="M40" t="n">
-        <v>0.1428571428571428</v>
+        <v>0.3548387096774193</v>
       </c>
       <c r="N40" t="n">
-        <v>1.101215362548828</v>
+        <v>10.23899173736572</v>
       </c>
       <c r="O40" t="n">
-        <v>1436.5625</v>
+        <v>1443.63671875</v>
       </c>
       <c r="P40" t="n">
-        <v>8.9</v>
+        <v>13.1</v>
       </c>
       <c r="Q40" t="n">
         <v>0</v>
@@ -3061,10 +3139,10 @@
         <v>0</v>
       </c>
       <c r="S40" t="n">
-        <v>0.04960846900939941</v>
+        <v>0.2441120147705078</v>
       </c>
       <c r="T40" t="n">
-        <v>1.051604509353638</v>
+        <v>9.994876861572266</v>
       </c>
       <c r="U40" t="n">
         <v>0</v>
@@ -3080,44 +3158,46 @@
         </is>
       </c>
       <c r="C41" t="n">
-        <v>0</v>
+        <v>0.2462462426271316</v>
       </c>
       <c r="D41" t="n">
-        <v>0</v>
+        <v>0.003115038339575822</v>
       </c>
       <c r="E41" t="n">
-        <v>0.2983242273330688</v>
+        <v>0.5215330123901367</v>
       </c>
       <c r="F41" t="n">
-        <v>-6.694999999999993</v>
+        <v>59.70530000000002</v>
       </c>
       <c r="G41" t="n">
-        <v>0.05349794238683128</v>
+        <v>0.3244170096021948</v>
       </c>
       <c r="H41" t="n">
-        <v>0</v>
+        <v>0.4</v>
       </c>
       <c r="I41" t="n">
         <v>1</v>
       </c>
-      <c r="J41" t="inlineStr"/>
+      <c r="J41" t="n">
+        <v>1</v>
+      </c>
       <c r="K41" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="L41" t="n">
-        <v>0.25</v>
+        <v>0.2647058823529412</v>
       </c>
       <c r="M41" t="n">
-        <v>0.1428571428571428</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="N41" t="n">
-        <v>0.4448699951171875</v>
+        <v>13.77950930595398</v>
       </c>
       <c r="O41" t="n">
-        <v>1436.5625</v>
+        <v>1443.64453125</v>
       </c>
       <c r="P41" t="n">
-        <v>9.199999999999999</v>
+        <v>13.6</v>
       </c>
       <c r="Q41" t="n">
         <v>0</v>
@@ -3126,10 +3206,10 @@
         <v>0</v>
       </c>
       <c r="S41" t="n">
-        <v>0.05235671997070312</v>
+        <v>0.239856481552124</v>
       </c>
       <c r="T41" t="n">
-        <v>0.3925108909606934</v>
+        <v>13.53964972496033</v>
       </c>
       <c r="U41" t="n">
         <v>0</v>
@@ -3145,44 +3225,46 @@
         </is>
       </c>
       <c r="C42" t="n">
-        <v>0.01273885288652687</v>
+        <v>0.215246632430976</v>
       </c>
       <c r="D42" t="n">
-        <v>7.842246496009318e-255</v>
+        <v>2.337053317910161e-79</v>
       </c>
       <c r="E42" t="n">
-        <v>0.3304620385169983</v>
+        <v>0.6265702843666077</v>
       </c>
       <c r="F42" t="n">
-        <v>-6.694999999999993</v>
+        <v>55.59536512027492</v>
       </c>
       <c r="G42" t="n">
-        <v>0.08914285714285715</v>
+        <v>0.4788571428571429</v>
       </c>
       <c r="H42" t="n">
-        <v>0</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="I42" t="n">
         <v>1</v>
       </c>
-      <c r="J42" t="inlineStr"/>
+      <c r="J42" t="n">
+        <v>1</v>
+      </c>
       <c r="K42" t="n">
         <v>0.5</v>
       </c>
       <c r="L42" t="n">
+        <v>0.2857142857142857</v>
+      </c>
+      <c r="M42" t="n">
         <v>0.25</v>
       </c>
-      <c r="M42" t="n">
-        <v>0.1428571428571428</v>
-      </c>
       <c r="N42" t="n">
-        <v>1.408112525939941</v>
+        <v>8.499035835266113</v>
       </c>
       <c r="O42" t="n">
-        <v>1436.5625</v>
+        <v>1443.64453125</v>
       </c>
       <c r="P42" t="n">
-        <v>8.9</v>
+        <v>11.9</v>
       </c>
       <c r="Q42" t="n">
         <v>0</v>
@@ -3191,10 +3273,10 @@
         <v>0</v>
       </c>
       <c r="S42" t="n">
-        <v>0.04854369163513184</v>
+        <v>0.2434766292572021</v>
       </c>
       <c r="T42" t="n">
-        <v>1.359566211700439</v>
+        <v>8.255556344985962</v>
       </c>
       <c r="U42" t="n">
         <v>0</v>
@@ -3210,44 +3292,46 @@
         </is>
       </c>
       <c r="C43" t="n">
-        <v>0</v>
+        <v>0.2238805923758076</v>
       </c>
       <c r="D43" t="n">
-        <v>0</v>
+        <v>0.02769771884910523</v>
       </c>
       <c r="E43" t="n">
-        <v>0.3637755811214447</v>
+        <v>0.6200291514396667</v>
       </c>
       <c r="F43" t="n">
-        <v>-6.694999999999993</v>
+        <v>24.72375</v>
       </c>
       <c r="G43" t="n">
-        <v>0.07228915662650602</v>
+        <v>0.556997219647822</v>
       </c>
       <c r="H43" t="n">
         <v>0</v>
       </c>
       <c r="I43" t="n">
-        <v>0</v>
-      </c>
-      <c r="J43" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J43" t="n">
+        <v>0</v>
+      </c>
       <c r="K43" t="n">
         <v>1</v>
       </c>
       <c r="L43" t="n">
-        <v>0.25</v>
+        <v>0.2875</v>
       </c>
       <c r="M43" t="n">
-        <v>0.02564102564102564</v>
+        <v>0.1372549019607843</v>
       </c>
       <c r="N43" t="n">
-        <v>1.95990252494812</v>
+        <v>12.3998806476593</v>
       </c>
       <c r="O43" t="n">
-        <v>1436.5703125</v>
+        <v>1443.64453125</v>
       </c>
       <c r="P43" t="n">
-        <v>9.300000000000001</v>
+        <v>14.3</v>
       </c>
       <c r="Q43" t="n">
         <v>0</v>
@@ -3256,10 +3340,10 @@
         <v>0</v>
       </c>
       <c r="S43" t="n">
-        <v>0.04887628555297852</v>
+        <v>0.2498202323913574</v>
       </c>
       <c r="T43" t="n">
-        <v>1.911023616790771</v>
+        <v>12.15005803108215</v>
       </c>
       <c r="U43" t="n">
         <v>0</v>
@@ -3275,19 +3359,19 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>0</v>
+        <v>0.1916666623697918</v>
       </c>
       <c r="D44" t="n">
-        <v>0</v>
+        <v>0.02872767822183733</v>
       </c>
       <c r="E44" t="n">
-        <v>0.3320682942867279</v>
+        <v>0.6812066435813904</v>
       </c>
       <c r="F44" t="n">
-        <v>-6.694999999999993</v>
+        <v>32.76696078431374</v>
       </c>
       <c r="G44" t="n">
-        <v>0.08955223880597014</v>
+        <v>0.5040183696900115</v>
       </c>
       <c r="H44" t="n">
         <v>0</v>
@@ -3295,24 +3379,26 @@
       <c r="I44" t="n">
         <v>0</v>
       </c>
-      <c r="J44" t="inlineStr"/>
+      <c r="J44" t="n">
+        <v>0</v>
+      </c>
       <c r="K44" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="L44" t="n">
-        <v>0.25</v>
+        <v>0.3275862068965517</v>
       </c>
       <c r="M44" t="n">
-        <v>0.07692307692307693</v>
+        <v>0.2307692307692308</v>
       </c>
       <c r="N44" t="n">
-        <v>0.3958652019500732</v>
+        <v>9.906358003616333</v>
       </c>
       <c r="O44" t="n">
-        <v>1436.66796875</v>
+        <v>1443.64453125</v>
       </c>
       <c r="P44" t="n">
-        <v>8.800000000000001</v>
+        <v>12.5</v>
       </c>
       <c r="Q44" t="n">
         <v>0</v>
@@ -3321,10 +3407,10 @@
         <v>0</v>
       </c>
       <c r="S44" t="n">
-        <v>0.04761886596679688</v>
+        <v>0.2687423229217529</v>
       </c>
       <c r="T44" t="n">
-        <v>0.348236083984375</v>
+        <v>9.637613296508789</v>
       </c>
       <c r="U44" t="n">
         <v>0</v>
@@ -3340,44 +3426,46 @@
         </is>
       </c>
       <c r="C45" t="n">
-        <v>0</v>
+        <v>0.1232394348990776</v>
       </c>
       <c r="D45" t="n">
-        <v>0</v>
+        <v>1.012019744289022e-162</v>
       </c>
       <c r="E45" t="n">
-        <v>0.3620854616165161</v>
+        <v>0.5612558722496033</v>
       </c>
       <c r="F45" t="n">
-        <v>-6.694999999999993</v>
+        <v>19.33928767123288</v>
       </c>
       <c r="G45" t="n">
-        <v>0.02138744173293118</v>
+        <v>0.08774335069920483</v>
       </c>
       <c r="H45" t="n">
-        <v>0</v>
+        <v>0.125</v>
       </c>
       <c r="I45" t="n">
         <v>0</v>
       </c>
-      <c r="J45" t="inlineStr"/>
+      <c r="J45" t="n">
+        <v>0</v>
+      </c>
       <c r="K45" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="L45" t="n">
-        <v>0.25</v>
+        <v>0.3260869565217391</v>
       </c>
       <c r="M45" t="n">
-        <v>0.07692307692307693</v>
+        <v>0.1397849462365592</v>
       </c>
       <c r="N45" t="n">
-        <v>1.395802974700928</v>
+        <v>11.77480959892273</v>
       </c>
       <c r="O45" t="n">
-        <v>1436.84765625</v>
+        <v>1443.734375</v>
       </c>
       <c r="P45" t="n">
-        <v>9.199999999999999</v>
+        <v>14.1</v>
       </c>
       <c r="Q45" t="n">
         <v>0</v>
@@ -3386,10 +3474,10 @@
         <v>0</v>
       </c>
       <c r="S45" t="n">
-        <v>0.04942727088928223</v>
+        <v>0.2444148063659668</v>
       </c>
       <c r="T45" t="n">
-        <v>1.346372842788696</v>
+        <v>11.53039193153381</v>
       </c>
       <c r="U45" t="n">
         <v>0</v>
@@ -3405,44 +3493,46 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>0</v>
+        <v>0.1900452459622039</v>
       </c>
       <c r="D46" t="n">
-        <v>0</v>
+        <v>0.0008419932130876846</v>
       </c>
       <c r="E46" t="n">
-        <v>0.3481395244598389</v>
+        <v>0.6237825155258179</v>
       </c>
       <c r="F46" t="n">
-        <v>-6.694999999999993</v>
+        <v>55.09198679471791</v>
       </c>
       <c r="G46" t="n">
-        <v>0.02160066463583495</v>
+        <v>0.198283024093049</v>
       </c>
       <c r="H46" t="n">
-        <v>0</v>
+        <v>0.3571428571428572</v>
       </c>
       <c r="I46" t="n">
-        <v>0</v>
-      </c>
-      <c r="J46" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J46" t="n">
+        <v>1</v>
+      </c>
       <c r="K46" t="n">
-        <v>0.3333333333333333</v>
+        <v>0.5</v>
       </c>
       <c r="L46" t="n">
-        <v>0.25</v>
+        <v>0.2929292929292929</v>
       </c>
       <c r="M46" t="n">
-        <v>0.1428571428571428</v>
+        <v>0.3805309734513274</v>
       </c>
       <c r="N46" t="n">
-        <v>1.423894643783569</v>
+        <v>19.91411447525024</v>
       </c>
       <c r="O46" t="n">
-        <v>1436.890625</v>
+        <v>1443.78125</v>
       </c>
       <c r="P46" t="n">
-        <v>10.5</v>
+        <v>15.1</v>
       </c>
       <c r="Q46" t="n">
         <v>0</v>
@@ -3451,10 +3541,10 @@
         <v>0</v>
       </c>
       <c r="S46" t="n">
-        <v>0.04790472984313965</v>
+        <v>0.285128116607666</v>
       </c>
       <c r="T46" t="n">
-        <v>1.375987529754639</v>
+        <v>19.62898397445679</v>
       </c>
       <c r="U46" t="n">
         <v>0</v>
@@ -3470,44 +3560,46 @@
         </is>
       </c>
       <c r="C47" t="n">
-        <v>0</v>
+        <v>0.2260869536201323</v>
       </c>
       <c r="D47" t="n">
-        <v>0</v>
+        <v>9.627878809907659e-81</v>
       </c>
       <c r="E47" t="n">
-        <v>0.3639097213745117</v>
+        <v>0.6099787950515747</v>
       </c>
       <c r="F47" t="n">
-        <v>-6.694999999999993</v>
+        <v>39.87156125608141</v>
       </c>
       <c r="G47" t="n">
-        <v>0.0310880829015544</v>
+        <v>0.2088481466719809</v>
       </c>
       <c r="H47" t="n">
-        <v>0</v>
+        <v>0.4285714285714285</v>
       </c>
       <c r="I47" t="n">
-        <v>0</v>
-      </c>
-      <c r="J47" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J47" t="n">
+        <v>1</v>
+      </c>
       <c r="K47" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="L47" t="n">
-        <v>0.25</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="M47" t="n">
-        <v>0.09090909090909091</v>
+        <v>0.2473118279569892</v>
       </c>
       <c r="N47" t="n">
-        <v>1.937818765640259</v>
+        <v>19.87475156784058</v>
       </c>
       <c r="O47" t="n">
-        <v>1436.8984375</v>
+        <v>1443.91796875</v>
       </c>
       <c r="P47" t="n">
-        <v>18.1</v>
+        <v>12.7</v>
       </c>
       <c r="Q47" t="n">
         <v>0</v>
@@ -3516,10 +3608,10 @@
         <v>0</v>
       </c>
       <c r="S47" t="n">
-        <v>0.04979729652404785</v>
+        <v>0.2409555912017822</v>
       </c>
       <c r="T47" t="n">
-        <v>1.888018846511841</v>
+        <v>19.63379287719727</v>
       </c>
       <c r="U47" t="n">
         <v>0</v>
@@ -3535,44 +3627,46 @@
         </is>
       </c>
       <c r="C48" t="n">
-        <v>0</v>
+        <v>0.2061855636178128</v>
       </c>
       <c r="D48" t="n">
-        <v>0</v>
+        <v>0.01269830595365195</v>
       </c>
       <c r="E48" t="n">
-        <v>0.3680242300033569</v>
+        <v>0.609144389629364</v>
       </c>
       <c r="F48" t="n">
-        <v>-6.694999999999993</v>
+        <v>35.70947058823532</v>
       </c>
       <c r="G48" t="n">
-        <v>0.1670235546038544</v>
+        <v>0.4047109207708779</v>
       </c>
       <c r="H48" t="n">
         <v>0</v>
       </c>
       <c r="I48" t="n">
-        <v>0</v>
-      </c>
-      <c r="J48" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J48" t="n">
+        <v>1</v>
+      </c>
       <c r="K48" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="L48" t="n">
-        <v>0.25</v>
+        <v>0.3125</v>
       </c>
       <c r="M48" t="n">
-        <v>0.07692307692307693</v>
+        <v>0.1666666666666667</v>
       </c>
       <c r="N48" t="n">
-        <v>0.261324405670166</v>
+        <v>18.18504762649536</v>
       </c>
       <c r="O48" t="n">
-        <v>1436.90234375</v>
+        <v>1443.99609375</v>
       </c>
       <c r="P48" t="n">
-        <v>18</v>
+        <v>15.4</v>
       </c>
       <c r="Q48" t="n">
         <v>0</v>
@@ -3581,10 +3675,10 @@
         <v>0</v>
       </c>
       <c r="S48" t="n">
-        <v>0.04862666130065918</v>
+        <v>0.2447407245635986</v>
       </c>
       <c r="T48" t="n">
-        <v>0.2126944065093994</v>
+        <v>17.94030427932739</v>
       </c>
       <c r="U48" t="n">
         <v>0</v>
@@ -3600,44 +3694,46 @@
         </is>
       </c>
       <c r="C49" t="n">
-        <v>0</v>
+        <v>0.1925925880537724</v>
       </c>
       <c r="D49" t="n">
-        <v>0</v>
+        <v>6.441354551294798e-79</v>
       </c>
       <c r="E49" t="n">
-        <v>0.3522202372550964</v>
+        <v>0.6491268873214722</v>
       </c>
       <c r="F49" t="n">
-        <v>-6.694999999999993</v>
+        <v>42.95500000000001</v>
       </c>
       <c r="G49" t="n">
-        <v>0.1502890173410405</v>
+        <v>0.6782273603082851</v>
       </c>
       <c r="H49" t="n">
-        <v>0</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="I49" t="n">
-        <v>0</v>
-      </c>
-      <c r="J49" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J49" t="n">
+        <v>1</v>
+      </c>
       <c r="K49" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="L49" t="n">
-        <v>0.25</v>
+        <v>0.2647058823529412</v>
       </c>
       <c r="M49" t="n">
-        <v>0.07692307692307693</v>
+        <v>0.178743961352657</v>
       </c>
       <c r="N49" t="n">
-        <v>2.098782300949097</v>
+        <v>17.59465980529785</v>
       </c>
       <c r="O49" t="n">
-        <v>1436.9140625</v>
+        <v>1444.0234375</v>
       </c>
       <c r="P49" t="n">
-        <v>11.5</v>
+        <v>13.9</v>
       </c>
       <c r="Q49" t="n">
         <v>0</v>
@@ -3646,10 +3742,10 @@
         <v>0</v>
       </c>
       <c r="S49" t="n">
-        <v>0.04910969734191895</v>
+        <v>0.2433815002441406</v>
       </c>
       <c r="T49" t="n">
-        <v>2.049670219421387</v>
+        <v>17.3512761592865</v>
       </c>
       <c r="U49" t="n">
         <v>0</v>
@@ -3665,44 +3761,46 @@
         </is>
       </c>
       <c r="C50" t="n">
-        <v>0</v>
+        <v>0.3195266222275131</v>
       </c>
       <c r="D50" t="n">
-        <v>0</v>
+        <v>1.573355140088374e-78</v>
       </c>
       <c r="E50" t="n">
-        <v>0.3514077365398407</v>
+        <v>0.6513027548789978</v>
       </c>
       <c r="F50" t="n">
-        <v>-6.694999999999993</v>
+        <v>45.32678160919542</v>
       </c>
       <c r="G50" t="n">
-        <v>0.1494252873563219</v>
+        <v>0.9885057471264368</v>
       </c>
       <c r="H50" t="n">
-        <v>0</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="I50" t="n">
-        <v>0</v>
-      </c>
-      <c r="J50" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J50" t="n">
+        <v>1</v>
+      </c>
       <c r="K50" t="n">
-        <v>0.5</v>
+        <v>0.75</v>
       </c>
       <c r="L50" t="n">
-        <v>0.25</v>
+        <v>0.3823529411764706</v>
       </c>
       <c r="M50" t="n">
-        <v>0.07692307692307693</v>
+        <v>0.2528735632183908</v>
       </c>
       <c r="N50" t="n">
-        <v>1.033989906311035</v>
+        <v>19.64222168922424</v>
       </c>
       <c r="O50" t="n">
-        <v>1436.9140625</v>
+        <v>1444.078125</v>
       </c>
       <c r="P50" t="n">
-        <v>9</v>
+        <v>13.9</v>
       </c>
       <c r="Q50" t="n">
         <v>0</v>
@@ -3711,10 +3809,10 @@
         <v>0</v>
       </c>
       <c r="S50" t="n">
-        <v>0.04962921142578125</v>
+        <v>0.2394795417785645</v>
       </c>
       <c r="T50" t="n">
-        <v>0.9843583106994629</v>
+        <v>19.40273952484131</v>
       </c>
       <c r="U50" t="n">
         <v>0</v>
@@ -3730,44 +3828,46 @@
         </is>
       </c>
       <c r="C51" t="n">
-        <v>0</v>
+        <v>0.3278688474593524</v>
       </c>
       <c r="D51" t="n">
-        <v>0</v>
+        <v>0.03185554685144382</v>
       </c>
       <c r="E51" t="n">
-        <v>0.3513664901256561</v>
+        <v>0.6248700022697449</v>
       </c>
       <c r="F51" t="n">
-        <v>-6.694999999999993</v>
+        <v>39.15545517241384</v>
       </c>
       <c r="G51" t="n">
-        <v>0.103861517976032</v>
+        <v>1.049267643142477</v>
       </c>
       <c r="H51" t="n">
-        <v>0</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="I51" t="n">
-        <v>0</v>
-      </c>
-      <c r="J51" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J51" t="n">
+        <v>1</v>
+      </c>
       <c r="K51" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="L51" t="n">
-        <v>0.25</v>
+        <v>0.2727272727272727</v>
       </c>
       <c r="M51" t="n">
-        <v>0.09090909090909091</v>
+        <v>0.3809523809523809</v>
       </c>
       <c r="N51" t="n">
-        <v>1.111335754394531</v>
+        <v>21.14945268630981</v>
       </c>
       <c r="O51" t="n">
-        <v>1436.91796875</v>
+        <v>1444.1015625</v>
       </c>
       <c r="P51" t="n">
-        <v>9.199999999999999</v>
+        <v>14.3</v>
       </c>
       <c r="Q51" t="n">
         <v>0</v>
@@ -3776,10 +3876,10 @@
         <v>0</v>
       </c>
       <c r="S51" t="n">
-        <v>0.04832911491394043</v>
+        <v>0.2385873794555664</v>
       </c>
       <c r="T51" t="n">
-        <v>1.063004016876221</v>
+        <v>20.91086292266846</v>
       </c>
       <c r="U51" t="n">
         <v>0</v>
@@ -3795,44 +3895,46 @@
         </is>
       </c>
       <c r="C52" t="n">
-        <v>0.008403360933196829</v>
+        <v>0.1868512079481807</v>
       </c>
       <c r="D52" t="n">
-        <v>2.960553565183628e-265</v>
+        <v>4.84516557083318e-157</v>
       </c>
       <c r="E52" t="n">
-        <v>0.3619620203971863</v>
+        <v>0.5342695713043213</v>
       </c>
       <c r="F52" t="n">
-        <v>-6.694999999999993</v>
+        <v>33.09357142857144</v>
       </c>
       <c r="G52" t="n">
-        <v>0.05656272661348803</v>
+        <v>0.2487309644670051</v>
       </c>
       <c r="H52" t="n">
-        <v>0</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="I52" t="n">
         <v>0</v>
       </c>
-      <c r="J52" t="inlineStr"/>
+      <c r="J52" t="n">
+        <v>1</v>
+      </c>
       <c r="K52" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="L52" t="n">
-        <v>0.25</v>
+        <v>0.2040816326530612</v>
       </c>
       <c r="M52" t="n">
-        <v>0.1111111111111111</v>
+        <v>0.1566265060240964</v>
       </c>
       <c r="N52" t="n">
-        <v>1.403618097305298</v>
+        <v>12.17007875442505</v>
       </c>
       <c r="O52" t="n">
-        <v>1436.921875</v>
+        <v>1444.109375</v>
       </c>
       <c r="P52" t="n">
-        <v>9.199999999999999</v>
+        <v>13.6</v>
       </c>
       <c r="Q52" t="n">
         <v>0</v>
@@ -3841,10 +3943,10 @@
         <v>0</v>
       </c>
       <c r="S52" t="n">
-        <v>0.05118560791015625</v>
+        <v>0.2423415184020996</v>
       </c>
       <c r="T52" t="n">
-        <v>1.352430105209351</v>
+        <v>11.92773461341858</v>
       </c>
       <c r="U52" t="n">
         <v>0</v>
@@ -3860,44 +3962,46 @@
         </is>
       </c>
       <c r="C53" t="n">
-        <v>0</v>
+        <v>0.3801295849631243</v>
       </c>
       <c r="D53" t="n">
-        <v>0</v>
+        <v>0.05221164602881641</v>
       </c>
       <c r="E53" t="n">
-        <v>0.3393140435218811</v>
+        <v>0.669135570526123</v>
       </c>
       <c r="F53" t="n">
-        <v>-6.694999999999993</v>
+        <v>46.60702172067357</v>
       </c>
       <c r="G53" t="n">
-        <v>0.0416221985058698</v>
+        <v>0.6558164354322306</v>
       </c>
       <c r="H53" t="n">
-        <v>0</v>
+        <v>0.7142857142857143</v>
       </c>
       <c r="I53" t="n">
-        <v>0</v>
-      </c>
-      <c r="J53" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J53" t="n">
+        <v>1</v>
+      </c>
       <c r="K53" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L53" t="n">
-        <v>0.25</v>
+        <v>0.3356164383561644</v>
       </c>
       <c r="M53" t="n">
-        <v>0.05263157894736842</v>
+        <v>0.5283018867924528</v>
       </c>
       <c r="N53" t="n">
-        <v>0.8527312278747559</v>
+        <v>27.76166749000549</v>
       </c>
       <c r="O53" t="n">
-        <v>1437.03125</v>
+        <v>1444.12890625</v>
       </c>
       <c r="P53" t="n">
-        <v>8.800000000000001</v>
+        <v>14.4</v>
       </c>
       <c r="Q53" t="n">
         <v>0</v>
@@ -3906,10 +4010,10 @@
         <v>0</v>
       </c>
       <c r="S53" t="n">
-        <v>0.04849863052368164</v>
+        <v>0.2384963035583496</v>
       </c>
       <c r="T53" t="n">
-        <v>0.8042299747467041</v>
+        <v>27.52316856384277</v>
       </c>
       <c r="U53" t="n">
         <v>0</v>
@@ -3925,44 +4029,46 @@
         </is>
       </c>
       <c r="C54" t="n">
-        <v>0</v>
+        <v>0.1610738212873295</v>
       </c>
       <c r="D54" t="n">
-        <v>0</v>
+        <v>6.357767916732833e-80</v>
       </c>
       <c r="E54" t="n">
-        <v>0.3256970345973969</v>
+        <v>0.6112699508666992</v>
       </c>
       <c r="F54" t="n">
-        <v>-6.694999999999993</v>
+        <v>-5.659957264957228</v>
       </c>
       <c r="G54" t="n">
-        <v>0.05739514348785872</v>
+        <v>0.4392935982339956</v>
       </c>
       <c r="H54" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I54" t="n">
-        <v>0</v>
-      </c>
-      <c r="J54" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J54" t="n">
+        <v>1</v>
+      </c>
       <c r="K54" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="L54" t="n">
-        <v>0.25</v>
+        <v>0.2142857142857143</v>
       </c>
       <c r="M54" t="n">
-        <v>0.07692307692307693</v>
+        <v>0.2857142857142857</v>
       </c>
       <c r="N54" t="n">
-        <v>0.4154658317565918</v>
+        <v>13.72128939628601</v>
       </c>
       <c r="O54" t="n">
-        <v>1437.0625</v>
+        <v>1444.18359375</v>
       </c>
       <c r="P54" t="n">
-        <v>9.199999999999999</v>
+        <v>14.1</v>
       </c>
       <c r="Q54" t="n">
         <v>0</v>
@@ -3971,10 +4077,10 @@
         <v>0</v>
       </c>
       <c r="S54" t="n">
-        <v>0.04831838607788086</v>
+        <v>0.243248462677002</v>
       </c>
       <c r="T54" t="n">
-        <v>0.3671443462371826</v>
+        <v>13.47803831100464</v>
       </c>
       <c r="U54" t="n">
         <v>0</v>
@@ -3990,44 +4096,46 @@
         </is>
       </c>
       <c r="C55" t="n">
-        <v>0</v>
+        <v>0.1678832092373062</v>
       </c>
       <c r="D55" t="n">
-        <v>0</v>
+        <v>6.524324042578614e-06</v>
       </c>
       <c r="E55" t="n">
-        <v>0.343548446893692</v>
+        <v>0.5519033670425415</v>
       </c>
       <c r="F55" t="n">
-        <v>-6.694999999999993</v>
+        <v>37.45538461538465</v>
       </c>
       <c r="G55" t="n">
-        <v>0.05045278137128072</v>
+        <v>0.165588615782665</v>
       </c>
       <c r="H55" t="n">
-        <v>0</v>
+        <v>0.1052631578947368</v>
       </c>
       <c r="I55" t="n">
-        <v>0</v>
-      </c>
-      <c r="J55" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J55" t="n">
+        <v>1</v>
+      </c>
       <c r="K55" t="n">
         <v>0.5</v>
       </c>
       <c r="L55" t="n">
-        <v>0.25</v>
+        <v>0.3636363636363636</v>
       </c>
       <c r="M55" t="n">
-        <v>0.1111111111111111</v>
+        <v>0.1463414634146341</v>
       </c>
       <c r="N55" t="n">
-        <v>0.9744696617126465</v>
+        <v>11.77563858032227</v>
       </c>
       <c r="O55" t="n">
-        <v>1437.15234375</v>
+        <v>1444.18359375</v>
       </c>
       <c r="P55" t="n">
-        <v>9</v>
+        <v>14.2</v>
       </c>
       <c r="Q55" t="n">
         <v>0</v>
@@ -4036,10 +4144,10 @@
         <v>0</v>
       </c>
       <c r="S55" t="n">
-        <v>0.05098199844360352</v>
+        <v>0.2531633377075195</v>
       </c>
       <c r="T55" t="n">
-        <v>0.9234855175018311</v>
+        <v>11.52247285842896</v>
       </c>
       <c r="U55" t="n">
         <v>0</v>
@@ -4061,13 +4169,13 @@
         <v>0</v>
       </c>
       <c r="E56" t="n">
-        <v>0.3342143893241882</v>
+        <v>0</v>
       </c>
       <c r="F56" t="n">
-        <v>-6.694999999999993</v>
+        <v>0</v>
       </c>
       <c r="G56" t="n">
-        <v>0.04977664326738992</v>
+        <v>0.02616464582003829</v>
       </c>
       <c r="H56" t="n">
         <v>0</v>
@@ -4077,22 +4185,22 @@
       </c>
       <c r="J56" t="inlineStr"/>
       <c r="K56" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="L56" t="n">
-        <v>0.25</v>
+        <v>0</v>
       </c>
       <c r="M56" t="n">
         <v>0.1111111111111111</v>
       </c>
       <c r="N56" t="n">
-        <v>1.484592914581299</v>
+        <v>4125.721278429031</v>
       </c>
       <c r="O56" t="n">
-        <v>1437.15234375</v>
+        <v>1449.90625</v>
       </c>
       <c r="P56" t="n">
-        <v>9.199999999999999</v>
+        <v>15</v>
       </c>
       <c r="Q56" t="n">
         <v>0</v>
@@ -4101,10 +4209,10 @@
         <v>0</v>
       </c>
       <c r="S56" t="n">
-        <v>0.05294489860534668</v>
+        <v>0.2388730049133301</v>
       </c>
       <c r="T56" t="n">
-        <v>1.43164587020874</v>
+        <v>4125.482402801514</v>
       </c>
       <c r="U56" t="n">
         <v>0</v>
@@ -4120,44 +4228,46 @@
         </is>
       </c>
       <c r="C57" t="n">
-        <v>0</v>
+        <v>0.2461059148106094</v>
       </c>
       <c r="D57" t="n">
-        <v>0</v>
+        <v>2.471901070465728e-79</v>
       </c>
       <c r="E57" t="n">
-        <v>0.3695140182971954</v>
+        <v>0.6101638078689575</v>
       </c>
       <c r="F57" t="n">
-        <v>-6.694999999999993</v>
+        <v>24.90221861471866</v>
       </c>
       <c r="G57" t="n">
-        <v>0.02687801516195727</v>
+        <v>0.4390075809786354</v>
       </c>
       <c r="H57" t="n">
-        <v>0</v>
+        <v>0.9166666666666666</v>
       </c>
       <c r="I57" t="n">
-        <v>0</v>
-      </c>
-      <c r="J57" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J57" t="n">
+        <v>1</v>
+      </c>
       <c r="K57" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="L57" t="n">
-        <v>0.25</v>
+        <v>0.225</v>
       </c>
       <c r="M57" t="n">
-        <v>0.04</v>
+        <v>0.3827160493827161</v>
       </c>
       <c r="N57" t="n">
-        <v>1.104376792907715</v>
+        <v>47.87333703041077</v>
       </c>
       <c r="O57" t="n">
-        <v>1437.171875</v>
+        <v>1449.90625</v>
       </c>
       <c r="P57" t="n">
-        <v>9.199999999999999</v>
+        <v>14.4</v>
       </c>
       <c r="Q57" t="n">
         <v>0</v>
@@ -4166,10 +4276,10 @@
         <v>0</v>
       </c>
       <c r="S57" t="n">
-        <v>0.05675482749938965</v>
+        <v>1.301597833633423</v>
       </c>
       <c r="T57" t="n">
-        <v>1.047619342803955</v>
+        <v>46.57173633575439</v>
       </c>
       <c r="U57" t="n">
         <v>0</v>
@@ -4185,44 +4295,46 @@
         </is>
       </c>
       <c r="C58" t="n">
-        <v>0.0120481921868196</v>
+        <v>0.2452830138687157</v>
       </c>
       <c r="D58" t="n">
-        <v>3.542014107114671e-257</v>
+        <v>3.707332481493019e-155</v>
       </c>
       <c r="E58" t="n">
-        <v>0.3487640619277954</v>
+        <v>0.6791971325874329</v>
       </c>
       <c r="F58" t="n">
-        <v>-6.694999999999993</v>
+        <v>28.27533766233768</v>
       </c>
       <c r="G58" t="n">
-        <v>0.08423326133909287</v>
+        <v>1.120950323974082</v>
       </c>
       <c r="H58" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I58" t="n">
-        <v>0</v>
-      </c>
-      <c r="J58" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J58" t="n">
+        <v>1</v>
+      </c>
       <c r="K58" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="L58" t="n">
         <v>0.25</v>
       </c>
       <c r="M58" t="n">
-        <v>0.1428571428571428</v>
+        <v>0.393939393939394</v>
       </c>
       <c r="N58" t="n">
-        <v>0.4971168041229248</v>
+        <v>32.5991153717041</v>
       </c>
       <c r="O58" t="n">
-        <v>1437.171875</v>
+        <v>1449.90625</v>
       </c>
       <c r="P58" t="n">
-        <v>18.2</v>
+        <v>14.3</v>
       </c>
       <c r="Q58" t="n">
         <v>0</v>
@@ -4231,10 +4343,10 @@
         <v>0</v>
       </c>
       <c r="S58" t="n">
-        <v>0.05186247825622559</v>
+        <v>0.2399046421051025</v>
       </c>
       <c r="T58" t="n">
-        <v>0.4452519416809082</v>
+        <v>32.35920858383179</v>
       </c>
       <c r="U58" t="n">
         <v>0</v>
@@ -4250,44 +4362,46 @@
         </is>
       </c>
       <c r="C59" t="n">
-        <v>0</v>
+        <v>0.2135922283042701</v>
       </c>
       <c r="D59" t="n">
-        <v>0</v>
+        <v>2.022400060987183e-155</v>
       </c>
       <c r="E59" t="n">
-        <v>0.359289288520813</v>
+        <v>0.5963390469551086</v>
       </c>
       <c r="F59" t="n">
-        <v>-6.694999999999993</v>
+        <v>52.82705128205131</v>
       </c>
       <c r="G59" t="n">
-        <v>0.09848484848484848</v>
+        <v>0.6351010101010101</v>
       </c>
       <c r="H59" t="n">
-        <v>0</v>
+        <v>0.1428571428571428</v>
       </c>
       <c r="I59" t="n">
-        <v>0</v>
-      </c>
-      <c r="J59" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J59" t="n">
+        <v>1</v>
+      </c>
       <c r="K59" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="L59" t="n">
-        <v>0.25</v>
+        <v>0.2054794520547945</v>
       </c>
       <c r="M59" t="n">
-        <v>0.1111111111111111</v>
+        <v>0.4117647058823529</v>
       </c>
       <c r="N59" t="n">
-        <v>0.9193322658538818</v>
+        <v>21.63844180107117</v>
       </c>
       <c r="O59" t="n">
-        <v>1437.19140625</v>
+        <v>1449.90625</v>
       </c>
       <c r="P59" t="n">
-        <v>18.2</v>
+        <v>13.7</v>
       </c>
       <c r="Q59" t="n">
         <v>0</v>
@@ -4296,10 +4410,10 @@
         <v>0</v>
       </c>
       <c r="S59" t="n">
-        <v>0.04835367202758789</v>
+        <v>0.2755162715911865</v>
       </c>
       <c r="T59" t="n">
-        <v>0.8709759712219238</v>
+        <v>21.36292290687561</v>
       </c>
       <c r="U59" t="n">
         <v>0</v>
@@ -4315,44 +4429,46 @@
         </is>
       </c>
       <c r="C60" t="n">
-        <v>0.00446428549356267</v>
+        <v>0.203147348719794</v>
       </c>
       <c r="D60" t="n">
-        <v>8.265132997605698e-314</v>
+        <v>0.01220172814257362</v>
       </c>
       <c r="E60" t="n">
-        <v>0.3573783934116364</v>
+        <v>0.6206266283988953</v>
       </c>
       <c r="F60" t="n">
-        <v>-6.694999999999993</v>
+        <v>14.97697631980989</v>
       </c>
       <c r="G60" t="n">
-        <v>0.02725366876310273</v>
+        <v>0.6296296296296297</v>
       </c>
       <c r="H60" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I60" t="n">
-        <v>0</v>
-      </c>
-      <c r="J60" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J60" t="n">
+        <v>1</v>
+      </c>
       <c r="K60" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L60" t="n">
-        <v>0.25</v>
+        <v>0.1878172588832487</v>
       </c>
       <c r="M60" t="n">
-        <v>0.07692307692307693</v>
+        <v>0.4774346793349169</v>
       </c>
       <c r="N60" t="n">
-        <v>0.6531040668487549</v>
+        <v>52.88502764701843</v>
       </c>
       <c r="O60" t="n">
-        <v>1437.1953125</v>
+        <v>1449.90625</v>
       </c>
       <c r="P60" t="n">
-        <v>17.4</v>
+        <v>14.6</v>
       </c>
       <c r="Q60" t="n">
         <v>0</v>
@@ -4361,10 +4477,10 @@
         <v>0</v>
       </c>
       <c r="S60" t="n">
-        <v>0.05022883415222168</v>
+        <v>0.2716195583343506</v>
       </c>
       <c r="T60" t="n">
-        <v>0.6028733253479004</v>
+        <v>52.61340546607971</v>
       </c>
       <c r="U60" t="n">
         <v>0</v>
@@ -4380,44 +4496,46 @@
         </is>
       </c>
       <c r="C61" t="n">
-        <v>0</v>
+        <v>0.1759999964364801</v>
       </c>
       <c r="D61" t="n">
-        <v>0</v>
+        <v>2.208023144735344e-155</v>
       </c>
       <c r="E61" t="n">
-        <v>0.3793801069259644</v>
+        <v>0.4606733024120331</v>
       </c>
       <c r="F61" t="n">
-        <v>-6.694999999999993</v>
+        <v>54.98732605042017</v>
       </c>
       <c r="G61" t="n">
-        <v>0.3157894736842105</v>
+        <v>2.595141700404858</v>
       </c>
       <c r="H61" t="n">
         <v>1</v>
       </c>
       <c r="I61" t="n">
-        <v>0</v>
-      </c>
-      <c r="J61" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J61" t="n">
+        <v>1</v>
+      </c>
       <c r="K61" t="n">
         <v>1</v>
       </c>
       <c r="L61" t="n">
-        <v>0.25</v>
+        <v>0.3246753246753247</v>
       </c>
       <c r="M61" t="n">
-        <v>0.05882352941176471</v>
+        <v>0.3248945147679325</v>
       </c>
       <c r="N61" t="n">
-        <v>2.156737327575684</v>
+        <v>26.06328940391541</v>
       </c>
       <c r="O61" t="n">
-        <v>1437.2109375</v>
+        <v>1449.90625</v>
       </c>
       <c r="P61" t="n">
-        <v>13.4</v>
+        <v>14.7</v>
       </c>
       <c r="Q61" t="n">
         <v>0</v>
@@ -4426,10 +4544,10 @@
         <v>0</v>
       </c>
       <c r="S61" t="n">
-        <v>0.05083203315734863</v>
+        <v>0.2403631210327148</v>
       </c>
       <c r="T61" t="n">
-        <v>2.105902910232544</v>
+        <v>25.82292413711548</v>
       </c>
       <c r="U61" t="n">
         <v>0</v>
@@ -4445,44 +4563,46 @@
         </is>
       </c>
       <c r="C62" t="n">
-        <v>0</v>
+        <v>0.2480620105907098</v>
       </c>
       <c r="D62" t="n">
-        <v>0</v>
+        <v>0.03041493233714596</v>
       </c>
       <c r="E62" t="n">
-        <v>0.3254241049289703</v>
+        <v>0.61978679895401</v>
       </c>
       <c r="F62" t="n">
-        <v>-6.694999999999993</v>
+        <v>31.99792910447763</v>
       </c>
       <c r="G62" t="n">
-        <v>0.195</v>
+        <v>0.8475</v>
       </c>
       <c r="H62" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I62" t="n">
         <v>0</v>
       </c>
-      <c r="J62" t="inlineStr"/>
+      <c r="J62" t="n">
+        <v>1</v>
+      </c>
       <c r="K62" t="n">
         <v>1</v>
       </c>
       <c r="L62" t="n">
-        <v>0.25</v>
+        <v>0.3181818181818182</v>
       </c>
       <c r="M62" t="n">
-        <v>0.07692307692307693</v>
+        <v>0.1304347826086956</v>
       </c>
       <c r="N62" t="n">
-        <v>1.62215256690979</v>
+        <v>12.90255641937256</v>
       </c>
       <c r="O62" t="n">
-        <v>1437.21484375</v>
+        <v>1449.90625</v>
       </c>
       <c r="P62" t="n">
-        <v>9</v>
+        <v>12.6</v>
       </c>
       <c r="Q62" t="n">
         <v>0</v>
@@ -4491,10 +4611,10 @@
         <v>0</v>
       </c>
       <c r="S62" t="n">
-        <v>0.0482642650604248</v>
+        <v>0.2366228103637695</v>
       </c>
       <c r="T62" t="n">
-        <v>1.573885679244995</v>
+        <v>12.66593050956726</v>
       </c>
       <c r="U62" t="n">
         <v>0</v>
@@ -4510,44 +4630,46 @@
         </is>
       </c>
       <c r="C63" t="n">
-        <v>0</v>
+        <v>0.234234229430647</v>
       </c>
       <c r="D63" t="n">
-        <v>0</v>
+        <v>2.194555027898429e-155</v>
       </c>
       <c r="E63" t="n">
-        <v>0.3176030814647675</v>
+        <v>0.6234097480773926</v>
       </c>
       <c r="F63" t="n">
-        <v>-6.694999999999993</v>
+        <v>36.95215909090911</v>
       </c>
       <c r="G63" t="n">
-        <v>0.1087866108786611</v>
+        <v>0.7629009762900977</v>
       </c>
       <c r="H63" t="n">
-        <v>0</v>
+        <v>0.75</v>
       </c>
       <c r="I63" t="n">
-        <v>0</v>
-      </c>
-      <c r="J63" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J63" t="n">
+        <v>1</v>
+      </c>
       <c r="K63" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="L63" t="n">
-        <v>0.25</v>
+        <v>0.352112676056338</v>
       </c>
       <c r="M63" t="n">
-        <v>0.07692307692307693</v>
+        <v>0.2248062015503876</v>
       </c>
       <c r="N63" t="n">
-        <v>1.889605045318604</v>
+        <v>17.4331750869751</v>
       </c>
       <c r="O63" t="n">
-        <v>1437.28515625</v>
+        <v>1449.90625</v>
       </c>
       <c r="P63" t="n">
-        <v>9.5</v>
+        <v>14.7</v>
       </c>
       <c r="Q63" t="n">
         <v>0</v>
@@ -4556,10 +4678,10 @@
         <v>0</v>
       </c>
       <c r="S63" t="n">
-        <v>0.04846763610839844</v>
+        <v>0.2767863273620605</v>
       </c>
       <c r="T63" t="n">
-        <v>1.841134786605835</v>
+        <v>17.1563868522644</v>
       </c>
       <c r="U63" t="n">
         <v>0</v>
@@ -4575,44 +4697,46 @@
         </is>
       </c>
       <c r="C64" t="n">
-        <v>0</v>
+        <v>0.226804118801148</v>
       </c>
       <c r="D64" t="n">
-        <v>0</v>
+        <v>3.230620562952813e-155</v>
       </c>
       <c r="E64" t="n">
-        <v>0.3184672594070435</v>
+        <v>0.6041204333305359</v>
       </c>
       <c r="F64" t="n">
-        <v>-6.694999999999993</v>
+        <v>50.92322139303485</v>
       </c>
       <c r="G64" t="n">
-        <v>0.1278688524590164</v>
+        <v>0.8557377049180328</v>
       </c>
       <c r="H64" t="n">
-        <v>0</v>
+        <v>0.75</v>
       </c>
       <c r="I64" t="n">
-        <v>0</v>
-      </c>
-      <c r="J64" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J64" t="n">
+        <v>1</v>
+      </c>
       <c r="K64" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="L64" t="n">
-        <v>0.25</v>
+        <v>0.3013698630136986</v>
       </c>
       <c r="M64" t="n">
-        <v>0.07692307692307693</v>
+        <v>0.2307692307692307</v>
       </c>
       <c r="N64" t="n">
-        <v>1.396763563156128</v>
+        <v>20.41695928573608</v>
       </c>
       <c r="O64" t="n">
-        <v>1437.37109375</v>
+        <v>1449.90625</v>
       </c>
       <c r="P64" t="n">
-        <v>8.9</v>
+        <v>13.6</v>
       </c>
       <c r="Q64" t="n">
         <v>0</v>
@@ -4621,10 +4745,10 @@
         <v>0</v>
       </c>
       <c r="S64" t="n">
-        <v>0.04960274696350098</v>
+        <v>0.2439033985137939</v>
       </c>
       <c r="T64" t="n">
-        <v>1.347158193588257</v>
+        <v>20.17305374145508</v>
       </c>
       <c r="U64" t="n">
         <v>0</v>
@@ -4640,44 +4764,46 @@
         </is>
       </c>
       <c r="C65" t="n">
-        <v>0</v>
+        <v>0.2624999951531251</v>
       </c>
       <c r="D65" t="n">
-        <v>0</v>
+        <v>2.932777909177495e-155</v>
       </c>
       <c r="E65" t="n">
-        <v>0.3219119608402252</v>
+        <v>0.6280467510223389</v>
       </c>
       <c r="F65" t="n">
-        <v>-6.694999999999993</v>
+        <v>50.32833333333338</v>
       </c>
       <c r="G65" t="n">
-        <v>0.156312625250501</v>
+        <v>0.7615230460921844</v>
       </c>
       <c r="H65" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I65" t="n">
-        <v>0</v>
-      </c>
-      <c r="J65" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J65" t="n">
+        <v>1</v>
+      </c>
       <c r="K65" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="L65" t="n">
-        <v>0.25</v>
+        <v>0.3846153846153846</v>
       </c>
       <c r="M65" t="n">
-        <v>0.07692307692307693</v>
+        <v>0.1818181818181818</v>
       </c>
       <c r="N65" t="n">
-        <v>1.178769111633301</v>
+        <v>7.869426727294922</v>
       </c>
       <c r="O65" t="n">
-        <v>1437.37109375</v>
+        <v>1449.90625</v>
       </c>
       <c r="P65" t="n">
-        <v>9</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="Q65" t="n">
         <v>0</v>
@@ -4686,10 +4812,10 @@
         <v>0</v>
       </c>
       <c r="S65" t="n">
-        <v>0.0506138801574707</v>
+        <v>0.2371289730072021</v>
       </c>
       <c r="T65" t="n">
-        <v>1.128152370452881</v>
+        <v>7.632293224334717</v>
       </c>
       <c r="U65" t="n">
         <v>0</v>
@@ -4705,44 +4831,46 @@
         </is>
       </c>
       <c r="C66" t="n">
-        <v>0</v>
+        <v>0.2198952844691758</v>
       </c>
       <c r="D66" t="n">
-        <v>0</v>
+        <v>1.400153425506653e-79</v>
       </c>
       <c r="E66" t="n">
-        <v>0.3294911682605743</v>
+        <v>0.6040650010108948</v>
       </c>
       <c r="F66" t="n">
-        <v>-6.694999999999993</v>
+        <v>66.61068548387098</v>
       </c>
       <c r="G66" t="n">
-        <v>0.09786700125470514</v>
+        <v>0.3801756587202008</v>
       </c>
       <c r="H66" t="n">
-        <v>0</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="I66" t="n">
-        <v>0</v>
-      </c>
-      <c r="J66" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J66" t="n">
+        <v>1</v>
+      </c>
       <c r="K66" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L66" t="n">
-        <v>0.25</v>
+        <v>0.3714285714285714</v>
       </c>
       <c r="M66" t="n">
-        <v>0.07692307692307693</v>
+        <v>0.1891891891891892</v>
       </c>
       <c r="N66" t="n">
-        <v>1.558030128479004</v>
+        <v>12.87119054794312</v>
       </c>
       <c r="O66" t="n">
-        <v>1437.46875</v>
+        <v>1449.90625</v>
       </c>
       <c r="P66" t="n">
-        <v>8.9</v>
+        <v>14</v>
       </c>
       <c r="Q66" t="n">
         <v>0</v>
@@ -4751,10 +4879,10 @@
         <v>0</v>
       </c>
       <c r="S66" t="n">
-        <v>0.05485844612121582</v>
+        <v>0.4214663505554199</v>
       </c>
       <c r="T66" t="n">
-        <v>1.503169298171997</v>
+        <v>12.44972133636475</v>
       </c>
       <c r="U66" t="n">
         <v>0</v>
@@ -4770,44 +4898,46 @@
         </is>
       </c>
       <c r="C67" t="n">
-        <v>0</v>
+        <v>0.2542372831715025</v>
       </c>
       <c r="D67" t="n">
-        <v>0</v>
+        <v>9.709914888250491e-79</v>
       </c>
       <c r="E67" t="n">
-        <v>0.3287849128246307</v>
+        <v>0.6543359160423279</v>
       </c>
       <c r="F67" t="n">
-        <v>-6.694999999999993</v>
+        <v>46.10734265734266</v>
       </c>
       <c r="G67" t="n">
-        <v>0.1068493150684932</v>
+        <v>0.9027397260273973</v>
       </c>
       <c r="H67" t="n">
-        <v>0</v>
+        <v>0.75</v>
       </c>
       <c r="I67" t="n">
-        <v>0</v>
-      </c>
-      <c r="J67" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J67" t="n">
+        <v>1</v>
+      </c>
       <c r="K67" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="L67" t="n">
-        <v>0.25</v>
+        <v>0.4146341463414634</v>
       </c>
       <c r="M67" t="n">
-        <v>0.07692307692307693</v>
+        <v>0.2741935483870968</v>
       </c>
       <c r="N67" t="n">
-        <v>393.8291125297546</v>
+        <v>9.633788108825684</v>
       </c>
       <c r="O67" t="n">
-        <v>1438.1328125</v>
+        <v>1449.90625</v>
       </c>
       <c r="P67" t="n">
-        <v>11.2</v>
+        <v>14.2</v>
       </c>
       <c r="Q67" t="n">
         <v>0</v>
@@ -4816,10 +4946,10 @@
         <v>0</v>
       </c>
       <c r="S67" t="n">
-        <v>0.04901838302612305</v>
+        <v>0.2804958820343018</v>
       </c>
       <c r="T67" t="n">
-        <v>393.7800920009613</v>
+        <v>9.353290319442749</v>
       </c>
       <c r="U67" t="n">
         <v>0</v>
@@ -4835,44 +4965,46 @@
         </is>
       </c>
       <c r="C68" t="n">
-        <v>0</v>
+        <v>0.09523809377676999</v>
       </c>
       <c r="D68" t="n">
-        <v>0</v>
+        <v>1.502992793091532e-155</v>
       </c>
       <c r="E68" t="n">
-        <v>0.4152870178222656</v>
+        <v>0.4814099669456482</v>
       </c>
       <c r="F68" t="n">
-        <v>-6.694999999999993</v>
+        <v>37.07089673913046</v>
       </c>
       <c r="G68" t="n">
-        <v>0.6141732283464567</v>
+        <v>9.700787401574804</v>
       </c>
       <c r="H68" t="n">
         <v>0</v>
       </c>
       <c r="I68" t="n">
-        <v>0</v>
-      </c>
-      <c r="J68" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J68" t="n">
+        <v>1</v>
+      </c>
       <c r="K68" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="L68" t="n">
-        <v>0.25</v>
+        <v>0.2467532467532468</v>
       </c>
       <c r="M68" t="n">
-        <v>0.2</v>
+        <v>0.6685082872928176</v>
       </c>
       <c r="N68" t="n">
-        <v>3.380919456481934</v>
+        <v>26.1925208568573</v>
       </c>
       <c r="O68" t="n">
-        <v>1438.13671875</v>
+        <v>1449.90625</v>
       </c>
       <c r="P68" t="n">
-        <v>8.6</v>
+        <v>13.4</v>
       </c>
       <c r="Q68" t="n">
         <v>0</v>
@@ -4881,10 +5013,10 @@
         <v>0</v>
       </c>
       <c r="S68" t="n">
-        <v>0.3026533126831055</v>
+        <v>0.2756891250610352</v>
       </c>
       <c r="T68" t="n">
-        <v>3.0782630443573</v>
+        <v>25.91682982444763</v>
       </c>
       <c r="U68" t="n">
         <v>0</v>

</xml_diff>